<commit_message>
Set deliverable S1 two-week option to 190 h and 44,559 AUD
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016KmKbhNhfEuuXeBfiH8ZpM
</commit_message>
<xml_diff>
--- a/NMMP_Reductions_Nuclear_Pharma.xlsx
+++ b/NMMP_Reductions_Nuclear_Pharma.xlsx
@@ -80,7 +80,7 @@
     <t xml:space="preserve">Commercial discount</t>
   </si>
   <si>
-    <t xml:space="preserve">4% discount on everything IDOM invoices, applied after the other reductions (4,192,253 AUD × 4%). Not applied to Plan Safe or INVAP.</t>
+    <t xml:space="preserve">4% discount on everything IDOM invoices, applied after the other reductions (4,197,549 AUD × 4%). Not applied to Plan Safe or INVAP.</t>
   </si>
   <si>
     <t xml:space="preserve">All</t>
@@ -89,7 +89,7 @@
     <t xml:space="preserve">S1 deliverable adjustment</t>
   </si>
   <si>
-    <t xml:space="preserve">Safety Assurance Plan / Safety Integration Plan priced as two weeks of work: a single, unrevised issue in Stage 1 of 165 hours and 38,675 AUD (≈2.2 senior authors full time for ten working days). The Stage 2 update is removed. Original price 432,419 AUD − 38,675 AUD.</t>
+    <t xml:space="preserve">Safety Assurance Plan / Safety Integration Plan priced as two weeks of work: a single, unrevised issue in Stage 1 of 190 hours and 44,559 AUD (2.5 FTEs full time for two weeks). The Stage 2 update is removed. Original price 432,419 AUD − 44,559 AUD.</t>
   </si>
   <si>
     <t xml:space="preserve">S1</t>
@@ -862,7 +862,7 @@
         <v>18</v>
       </c>
       <c r="D5" s="5" t="n">
-        <v>167690.116377778</v>
+        <v>167901.940377778</v>
       </c>
       <c r="E5" s="6" t="s">
         <v>19</v>
@@ -888,7 +888,7 @@
         <v>21</v>
       </c>
       <c r="D6" s="5" t="n">
-        <v>393743.875</v>
+        <v>387859.875</v>
       </c>
       <c r="E6" s="6" t="s">
         <v>22</v>
@@ -1045,7 +1045,7 @@
       </c>
       <c r="D15" s="11" t="n">
         <f aca="false">SUM(D3:D7)</f>
-        <v>1929008.20443333</v>
+        <v>1923336.02843333</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1054,7 +1054,7 @@
       </c>
       <c r="D16" s="11" t="n">
         <f aca="false">SUM(D3:D8)</f>
-        <v>3150723.73443333</v>
+        <v>3145051.55843333</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1153,29 +1153,29 @@
         <v>335082.825</v>
       </c>
       <c r="C4" s="15" t="n">
-        <v>223637.064170136</v>
+        <v>229226.532693237</v>
       </c>
       <c r="D4" s="15" t="n">
-        <v>115570.014170136</v>
+        <v>121159.482693237</v>
       </c>
       <c r="E4" s="14" t="n">
         <v>106000</v>
       </c>
       <c r="F4" s="16" t="n">
         <f aca="false">IF(B4=0,0,1-C4/B4)</f>
-        <v>0.332591683354299</v>
+        <v>0.315910826843372</v>
       </c>
       <c r="G4" s="16" t="n">
         <f aca="false">IF(B4=0,0,1-D4/B4)</f>
-        <v>0.655100155699905</v>
+        <v>0.638419299188978</v>
       </c>
       <c r="H4" s="17" t="n">
         <f aca="false">IF(C4=0,0,(E4-C4)/C4)</f>
-        <v>-0.52601774489689</v>
+        <v>-0.537575346297914</v>
       </c>
       <c r="I4" s="17" t="n">
         <f aca="false">IF(D4=0,0,(E4-D4)/D4)</f>
-        <v>-0.0828070692805102</v>
+        <v>-0.125120067833396</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1186,29 +1186,29 @@
         <v>732839.1</v>
       </c>
       <c r="C5" s="15" t="n">
-        <v>294472.158412194</v>
+        <v>294474.780970431</v>
       </c>
       <c r="D5" s="15" t="n">
-        <v>135605.583412194</v>
+        <v>135608.205970431</v>
       </c>
       <c r="E5" s="14" t="n">
         <v>453000</v>
       </c>
       <c r="F5" s="16" t="n">
         <f aca="false">IF(B5=0,0,1-C5/B5)</f>
-        <v>0.598176245765006</v>
+        <v>0.598172667137396</v>
       </c>
       <c r="G5" s="16" t="n">
         <f aca="false">IF(B5=0,0,1-D5/B5)</f>
-        <v>0.814958585844841</v>
+        <v>0.814955007217231</v>
       </c>
       <c r="H5" s="17" t="n">
         <f aca="false">IF(C5=0,0,(E5-C5)/C5)</f>
-        <v>0.538345772458064</v>
+        <v>0.53833207212908</v>
       </c>
       <c r="I5" s="17" t="n">
         <f aca="false">IF(D5=0,0,(E5-D5)/D5)</f>
-        <v>2.34057041459006</v>
+        <v>2.34050581053167</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1219,29 +1219,29 @@
         <v>1469323.8</v>
       </c>
       <c r="C6" s="15" t="n">
-        <v>1138277.84394111</v>
+        <v>1138296.28283098</v>
       </c>
       <c r="D6" s="15" t="n">
-        <v>948471.443941112</v>
+        <v>948489.882830978</v>
       </c>
       <c r="E6" s="14" t="n">
         <v>1250000</v>
       </c>
       <c r="F6" s="16" t="n">
         <f aca="false">IF(B6=0,0,1-C6/B6)</f>
-        <v>0.225304970938938</v>
+        <v>0.225292421703793</v>
       </c>
       <c r="G6" s="16" t="n">
         <f aca="false">IF(B6=0,0,1-D6/B6)</f>
-        <v>0.354484393473303</v>
+        <v>0.35447184423816</v>
       </c>
       <c r="H6" s="17" t="n">
         <f aca="false">IF(C6=0,0,(E6-C6)/C6)</f>
-        <v>0.0981501631201653</v>
+        <v>0.0981323745441822</v>
       </c>
       <c r="I6" s="17" t="n">
         <f aca="false">IF(D6=0,0,(E6-D6)/D6)</f>
-        <v>0.317909999278385</v>
+        <v>0.317884378765431</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1252,29 +1252,29 @@
         <v>3183882.555</v>
       </c>
       <c r="C7" s="15" t="n">
-        <v>2447129.72312514</v>
+        <v>2447168.9820988</v>
       </c>
       <c r="D7" s="15" t="n">
-        <v>2014025.09312514</v>
+        <v>2014064.3520988</v>
       </c>
       <c r="E7" s="14" t="n">
         <v>1455000</v>
       </c>
       <c r="F7" s="16" t="n">
         <f aca="false">IF(B7=0,0,1-C7/B7)</f>
-        <v>0.231400756512785</v>
+        <v>0.231388425978294</v>
       </c>
       <c r="G7" s="16" t="n">
         <f aca="false">IF(B7=0,0,1-D7/B7)</f>
-        <v>0.367431097619384</v>
+        <v>0.367418767084893</v>
       </c>
       <c r="H7" s="17" t="n">
         <f aca="false">IF(C7=0,0,(E7-C7)/C7)</f>
-        <v>-0.405425880675475</v>
+        <v>-0.405435419195234</v>
       </c>
       <c r="I7" s="17" t="n">
         <f aca="false">IF(D7=0,0,(E7-D7)/D7)</f>
-        <v>-0.277566101352644</v>
+        <v>-0.277580183332382</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1285,29 +1285,29 @@
         <v>540610.875</v>
       </c>
       <c r="C8" s="15" t="n">
-        <v>284770.27415548</v>
+        <v>284773.170543182</v>
       </c>
       <c r="D8" s="15" t="n">
-        <v>156237.14915548</v>
+        <v>156240.045543182</v>
       </c>
       <c r="E8" s="14" t="n">
         <v>370000</v>
       </c>
       <c r="F8" s="16" t="n">
         <f aca="false">IF(B8=0,0,1-C8/B8)</f>
-        <v>0.473243533705311</v>
+        <v>0.473238176085189</v>
       </c>
       <c r="G8" s="16" t="n">
         <f aca="false">IF(B8=0,0,1-D8/B8)</f>
-        <v>0.710998878527037</v>
+        <v>0.710993520906915</v>
       </c>
       <c r="H8" s="17" t="n">
         <f aca="false">IF(C8=0,0,(E8-C8)/C8)</f>
-        <v>0.299292916359613</v>
+        <v>0.299279701434846</v>
       </c>
       <c r="I8" s="17" t="n">
         <f aca="false">IF(D8=0,0,(E8-D8)/D8)</f>
-        <v>1.36819477313807</v>
+        <v>1.36815087139576</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1318,29 +1318,29 @@
         <v>775079.55</v>
       </c>
       <c r="C9" s="15" t="n">
-        <v>742511.341496081</v>
+        <v>742522.76735156</v>
       </c>
       <c r="D9" s="15" t="n">
-        <v>595621.591496081</v>
+        <v>595633.01735156</v>
       </c>
       <c r="E9" s="14" t="n">
         <v>102000</v>
       </c>
       <c r="F9" s="16" t="n">
         <f aca="false">IF(B9=0,0,1-C9/B9)</f>
-        <v>0.0420191817780756</v>
+        <v>0.0420044402518943</v>
       </c>
       <c r="G9" s="16" t="n">
         <f aca="false">IF(B9=0,0,1-D9/B9)</f>
-        <v>0.23153489019794</v>
+        <v>0.231520148671759</v>
       </c>
       <c r="H9" s="17" t="n">
         <f aca="false">IF(C9=0,0,(E9-C9)/C9)</f>
-        <v>-0.862628360942634</v>
+        <v>-0.862630474801716</v>
       </c>
       <c r="I9" s="17" t="n">
         <f aca="false">IF(D9=0,0,(E9-D9)/D9)</f>
-        <v>-0.828750331659743</v>
+        <v>-0.82875361669248</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1351,29 +1351,29 @@
         <v>493905.3</v>
       </c>
       <c r="C10" s="15" t="n">
-        <v>470917.395266522</v>
+        <v>470925.460078476</v>
       </c>
       <c r="D10" s="15" t="n">
-        <v>414469.395266522</v>
+        <v>414477.460078476</v>
       </c>
       <c r="E10" s="14" t="n">
         <v>73000</v>
       </c>
       <c r="F10" s="16" t="n">
         <f aca="false">IF(B10=0,0,1-C10/B10)</f>
-        <v>0.0465431424475056</v>
+        <v>0.0465268137870235</v>
       </c>
       <c r="G10" s="16" t="n">
         <f aca="false">IF(B10=0,0,1-D10/B10)</f>
-        <v>0.160832258194998</v>
+        <v>0.160815929534516</v>
       </c>
       <c r="H10" s="17" t="n">
         <f aca="false">IF(C10=0,0,(E10-C10)/C10)</f>
-        <v>-0.844983428656984</v>
+        <v>-0.844986083386031</v>
       </c>
       <c r="I10" s="17" t="n">
         <f aca="false">IF(D10=0,0,(E10-D10)/D10)</f>
-        <v>-0.823871193304737</v>
+        <v>-0.823874620380615</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1386,11 +1386,11 @@
       </c>
       <c r="C11" s="19" t="n">
         <f aca="false">SUM(C4:C10)</f>
-        <v>5601715.80056666</v>
+        <v>5607387.97656667</v>
       </c>
       <c r="D11" s="19" t="n">
         <f aca="false">SUM(D4:D10)</f>
-        <v>4380000.27056667</v>
+        <v>4385672.44656666</v>
       </c>
       <c r="E11" s="19" t="n">
         <f aca="false">SUM(E4:E10)</f>
@@ -1398,19 +1398,19 @@
       </c>
       <c r="F11" s="20" t="n">
         <f aca="false">IF(B11=0,0,1-C11/B11)</f>
-        <v>0.256151759532361</v>
+        <v>0.255398554927301</v>
       </c>
       <c r="G11" s="20" t="n">
         <f aca="false">IF(B11=0,0,1-D11/B11)</f>
-        <v>0.418382579462668</v>
+        <v>0.417629374857609</v>
       </c>
       <c r="H11" s="21" t="n">
         <f aca="false">IF(C11=0,0,(E11-C11)/C11)</f>
-        <v>-0.320029766662799</v>
+        <v>-0.320717593304075</v>
       </c>
       <c r="I11" s="21" t="n">
         <f aca="false">IF(D11=0,0,(E11-D11)/D11)</f>
-        <v>-0.130365350523778</v>
+        <v>-0.131490085863141</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1684,11 +1684,11 @@
       </c>
       <c r="C28" s="15" t="n">
         <f aca="false">C4+D15</f>
-        <v>223637.064170136</v>
+        <v>229226.532693237</v>
       </c>
       <c r="D28" s="15" t="n">
         <f aca="false">D4+D15</f>
-        <v>115570.014170136</v>
+        <v>121159.482693237</v>
       </c>
       <c r="E28" s="14" t="n">
         <f aca="false">E4+N(E15)</f>
@@ -1696,19 +1696,19 @@
       </c>
       <c r="F28" s="16" t="n">
         <f aca="false">IF(B28=0,0,1-C28/B28)</f>
-        <v>0.332591683354299</v>
+        <v>0.315910826843372</v>
       </c>
       <c r="G28" s="16" t="n">
         <f aca="false">IF(B28=0,0,1-D28/B28)</f>
-        <v>0.655100155699905</v>
+        <v>0.638419299188978</v>
       </c>
       <c r="H28" s="17" t="n">
         <f aca="false">IF(C28=0,0,(E28-C28)/C28)</f>
-        <v>-0.52601774489689</v>
+        <v>-0.537575346297914</v>
       </c>
       <c r="I28" s="17" t="n">
         <f aca="false">IF(D28=0,0,(E28-D28)/D28)</f>
-        <v>-0.0828070692805102</v>
+        <v>-0.125120067833396</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1721,11 +1721,11 @@
       </c>
       <c r="C29" s="15" t="n">
         <f aca="false">C5+D16</f>
-        <v>294472.158412194</v>
+        <v>294474.780970431</v>
       </c>
       <c r="D29" s="15" t="n">
         <f aca="false">D5+D16</f>
-        <v>135605.583412194</v>
+        <v>135608.205970431</v>
       </c>
       <c r="E29" s="14" t="n">
         <f aca="false">E5+N(E16)</f>
@@ -1733,19 +1733,19 @@
       </c>
       <c r="F29" s="16" t="n">
         <f aca="false">IF(B29=0,0,1-C29/B29)</f>
-        <v>0.598176245765006</v>
+        <v>0.598172667137396</v>
       </c>
       <c r="G29" s="16" t="n">
         <f aca="false">IF(B29=0,0,1-D29/B29)</f>
-        <v>0.814958585844841</v>
+        <v>0.814955007217231</v>
       </c>
       <c r="H29" s="17" t="n">
         <f aca="false">IF(C29=0,0,(E29-C29)/C29)</f>
-        <v>0.538345772458064</v>
+        <v>0.53833207212908</v>
       </c>
       <c r="I29" s="17" t="n">
         <f aca="false">IF(D29=0,0,(E29-D29)/D29)</f>
-        <v>2.34057041459006</v>
+        <v>2.34050581053167</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1758,11 +1758,11 @@
       </c>
       <c r="C30" s="15" t="n">
         <f aca="false">C6+D17</f>
-        <v>1138277.84394111</v>
+        <v>1138296.28283098</v>
       </c>
       <c r="D30" s="15" t="n">
         <f aca="false">D6+D17</f>
-        <v>948471.443941112</v>
+        <v>948489.882830978</v>
       </c>
       <c r="E30" s="14" t="n">
         <f aca="false">E6+N(E17)</f>
@@ -1770,19 +1770,19 @@
       </c>
       <c r="F30" s="16" t="n">
         <f aca="false">IF(B30=0,0,1-C30/B30)</f>
-        <v>0.225304970938938</v>
+        <v>0.225292421703793</v>
       </c>
       <c r="G30" s="16" t="n">
         <f aca="false">IF(B30=0,0,1-D30/B30)</f>
-        <v>0.354484393473303</v>
+        <v>0.35447184423816</v>
       </c>
       <c r="H30" s="17" t="n">
         <f aca="false">IF(C30=0,0,(E30-C30)/C30)</f>
-        <v>0.0981501631201653</v>
+        <v>0.0981323745441822</v>
       </c>
       <c r="I30" s="17" t="n">
         <f aca="false">IF(D30=0,0,(E30-D30)/D30)</f>
-        <v>0.317909999278385</v>
+        <v>0.317884378765431</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1795,11 +1795,11 @@
       </c>
       <c r="C31" s="15" t="n">
         <f aca="false">C7+D18</f>
-        <v>2447129.72312514</v>
+        <v>2447168.9820988</v>
       </c>
       <c r="D31" s="15" t="n">
         <f aca="false">D7+D18</f>
-        <v>2014025.09312514</v>
+        <v>2014064.3520988</v>
       </c>
       <c r="E31" s="14" t="n">
         <f aca="false">E7+N(E18)</f>
@@ -1807,19 +1807,19 @@
       </c>
       <c r="F31" s="16" t="n">
         <f aca="false">IF(B31=0,0,1-C31/B31)</f>
-        <v>0.231400756512785</v>
+        <v>0.231388425978294</v>
       </c>
       <c r="G31" s="16" t="n">
         <f aca="false">IF(B31=0,0,1-D31/B31)</f>
-        <v>0.367431097619384</v>
+        <v>0.367418767084893</v>
       </c>
       <c r="H31" s="17" t="n">
         <f aca="false">IF(C31=0,0,(E31-C31)/C31)</f>
-        <v>-0.405425880675475</v>
+        <v>-0.405435419195234</v>
       </c>
       <c r="I31" s="17" t="n">
         <f aca="false">IF(D31=0,0,(E31-D31)/D31)</f>
-        <v>-0.277566101352644</v>
+        <v>-0.277580183332382</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1832,11 +1832,11 @@
       </c>
       <c r="C32" s="15" t="n">
         <f aca="false">C8+D19</f>
-        <v>284770.27415548</v>
+        <v>284773.170543182</v>
       </c>
       <c r="D32" s="15" t="n">
         <f aca="false">D8+D19</f>
-        <v>156237.14915548</v>
+        <v>156240.045543182</v>
       </c>
       <c r="E32" s="14" t="n">
         <f aca="false">E8+N(E19)</f>
@@ -1844,19 +1844,19 @@
       </c>
       <c r="F32" s="16" t="n">
         <f aca="false">IF(B32=0,0,1-C32/B32)</f>
-        <v>0.473243533705311</v>
+        <v>0.473238176085189</v>
       </c>
       <c r="G32" s="16" t="n">
         <f aca="false">IF(B32=0,0,1-D32/B32)</f>
-        <v>0.710998878527037</v>
+        <v>0.710993520906915</v>
       </c>
       <c r="H32" s="17" t="n">
         <f aca="false">IF(C32=0,0,(E32-C32)/C32)</f>
-        <v>0.299292916359613</v>
+        <v>0.299279701434846</v>
       </c>
       <c r="I32" s="17" t="n">
         <f aca="false">IF(D32=0,0,(E32-D32)/D32)</f>
-        <v>1.36819477313807</v>
+        <v>1.36815087139576</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1869,11 +1869,11 @@
       </c>
       <c r="C33" s="15" t="n">
         <f aca="false">C9+D20</f>
-        <v>742511.341496081</v>
+        <v>742522.76735156</v>
       </c>
       <c r="D33" s="15" t="n">
         <f aca="false">D9+D20</f>
-        <v>595621.591496081</v>
+        <v>595633.01735156</v>
       </c>
       <c r="E33" s="14" t="n">
         <f aca="false">E9+N(E20)</f>
@@ -1881,19 +1881,19 @@
       </c>
       <c r="F33" s="16" t="n">
         <f aca="false">IF(B33=0,0,1-C33/B33)</f>
-        <v>0.0420191817780756</v>
+        <v>0.0420044402518943</v>
       </c>
       <c r="G33" s="16" t="n">
         <f aca="false">IF(B33=0,0,1-D33/B33)</f>
-        <v>0.23153489019794</v>
+        <v>0.231520148671759</v>
       </c>
       <c r="H33" s="17" t="n">
         <f aca="false">IF(C33=0,0,(E33-C33)/C33)</f>
-        <v>-0.862628360942634</v>
+        <v>-0.862630474801716</v>
       </c>
       <c r="I33" s="17" t="n">
         <f aca="false">IF(D33=0,0,(E33-D33)/D33)</f>
-        <v>-0.828750331659743</v>
+        <v>-0.82875361669248</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1906,11 +1906,11 @@
       </c>
       <c r="C34" s="15" t="n">
         <f aca="false">C10+D21</f>
-        <v>470917.395266522</v>
+        <v>470925.460078476</v>
       </c>
       <c r="D34" s="15" t="n">
         <f aca="false">D10+D21</f>
-        <v>414469.395266522</v>
+        <v>414477.460078476</v>
       </c>
       <c r="E34" s="14" t="n">
         <f aca="false">E10+N(E21)</f>
@@ -1918,19 +1918,19 @@
       </c>
       <c r="F34" s="16" t="n">
         <f aca="false">IF(B34=0,0,1-C34/B34)</f>
-        <v>0.0465431424475056</v>
+        <v>0.0465268137870235</v>
       </c>
       <c r="G34" s="16" t="n">
         <f aca="false">IF(B34=0,0,1-D34/B34)</f>
-        <v>0.160832258194998</v>
+        <v>0.160815929534516</v>
       </c>
       <c r="H34" s="17" t="n">
         <f aca="false">IF(C34=0,0,(E34-C34)/C34)</f>
-        <v>-0.844983428656984</v>
+        <v>-0.844986083386031</v>
       </c>
       <c r="I34" s="17" t="n">
         <f aca="false">IF(D34=0,0,(E34-D34)/D34)</f>
-        <v>-0.823871193304737</v>
+        <v>-0.823874620380615</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1943,11 +1943,11 @@
       </c>
       <c r="C35" s="19" t="n">
         <f aca="false">SUM(C28:C34)</f>
-        <v>5601715.80056666</v>
+        <v>5607387.97656667</v>
       </c>
       <c r="D35" s="19" t="n">
         <f aca="false">SUM(D28:D34)</f>
-        <v>4380000.27056667</v>
+        <v>4385672.44656666</v>
       </c>
       <c r="E35" s="19" t="n">
         <f aca="false">SUM(E28:E34)</f>
@@ -1955,19 +1955,19 @@
       </c>
       <c r="F35" s="20" t="n">
         <f aca="false">IF(B35=0,0,1-C35/B35)</f>
-        <v>0.256151759532361</v>
+        <v>0.255398554927301</v>
       </c>
       <c r="G35" s="20" t="n">
         <f aca="false">IF(B35=0,0,1-D35/B35)</f>
-        <v>0.418382579462668</v>
+        <v>0.417629374857609</v>
       </c>
       <c r="H35" s="21" t="n">
         <f aca="false">IF(C35=0,0,(E35-C35)/C35)</f>
-        <v>-0.320029766662799</v>
+        <v>-0.320717593304075</v>
       </c>
       <c r="I35" s="21" t="n">
         <f aca="false">IF(D35=0,0,(E35-D35)/D35)</f>
-        <v>-0.130365350523778</v>
+        <v>-0.131490085863141</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2011,18 +2011,18 @@
         <v>5858217.9075</v>
       </c>
       <c r="C40" s="14" t="n">
-        <v>4024562.79306667</v>
+        <v>4029646.56906667</v>
       </c>
       <c r="D40" s="14" t="n">
-        <v>4024562.79306667</v>
+        <v>4029646.56906667</v>
       </c>
       <c r="E40" s="14" t="n">
         <f aca="false">B40-C40</f>
-        <v>1833655.11443333</v>
+        <v>1828571.33843333</v>
       </c>
       <c r="F40" s="14" t="n">
         <f aca="false">B40-D40</f>
-        <v>1833655.11443333</v>
+        <v>1828571.33843333</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2033,18 +2033,18 @@
         <v>1593669.9975</v>
       </c>
       <c r="C41" s="14" t="n">
-        <v>1498316.9075</v>
+        <v>1498905.3075</v>
       </c>
       <c r="D41" s="14" t="n">
-        <v>276601.3775</v>
+        <v>277189.7775</v>
       </c>
       <c r="E41" s="14" t="n">
         <f aca="false">B41-C41</f>
-        <v>95353.0900000001</v>
+        <v>94764.6899999999</v>
       </c>
       <c r="F41" s="14" t="n">
         <f aca="false">B41-D41</f>
-        <v>1317068.62</v>
+        <v>1316480.22</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2079,19 +2079,19 @@
       </c>
       <c r="C43" s="19" t="n">
         <f aca="false">SUM(C40:C42)</f>
-        <v>5601715.80056667</v>
+        <v>5607387.97656667</v>
       </c>
       <c r="D43" s="19" t="n">
         <f aca="false">SUM(D40:D42)</f>
-        <v>4380000.27056667</v>
+        <v>4385672.44656667</v>
       </c>
       <c r="E43" s="19" t="n">
         <f aca="false">SUM(E40:E42)</f>
-        <v>1929008.20443333</v>
+        <v>1923336.02843333</v>
       </c>
       <c r="F43" s="19" t="n">
         <f aca="false">SUM(F40:F42)</f>
-        <v>3150723.73443333</v>
+        <v>3145051.55843333</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Descope SSC deliverables in all stages (S1-S7)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016KmKbhNhfEuuXeBfiH8ZpM
</commit_message>
<xml_diff>
--- a/NMMP_Reductions_Nuclear_Pharma.xlsx
+++ b/NMMP_Reductions_Nuclear_Pharma.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="72">
   <si>
     <t xml:space="preserve">Reductions on the NMMP offer — all amounts in AUD. Nuclear reductions are applied in sequence, without double counting: SSC descoping → S1 deliverable adjustment → rework → travel → commercial discount. Plan Safe applies to Scenario 2 only.</t>
   </si>
@@ -74,13 +74,13 @@
     <t xml:space="preserve">S26, S27, S28, S29</t>
   </si>
   <si>
-    <t xml:space="preserve">S1-S5</t>
+    <t xml:space="preserve">S1-S7</t>
   </si>
   <si>
     <t xml:space="preserve">Commercial discount</t>
   </si>
   <si>
-    <t xml:space="preserve">4% discount on everything IDOM invoices, applied after the other reductions (4,197,549 AUD × 4%). Not applied to Plan Safe or INVAP.</t>
+    <t xml:space="preserve">4% discount on everything IDOM invoices, applied after the other reductions (3,817,908 AUD × 4%). Not applied to Plan Safe or INVAP.</t>
   </si>
   <si>
     <t xml:space="preserve">All</t>
@@ -105,9 +105,6 @@
   </si>
   <si>
     <t xml:space="preserve">S2, S3, S8, S30</t>
-  </si>
-  <si>
-    <t xml:space="preserve">S1-S7</t>
   </si>
   <si>
     <t xml:space="preserve">Scenario 2 only</t>
@@ -835,11 +832,11 @@
         <v>15</v>
       </c>
       <c r="D4" s="5" t="n">
-        <v>1250657.625</v>
+        <v>1652324.1</v>
       </c>
       <c r="E4" s="6" t="str">
-        <f aca="false">"SSC Categorisation Report (S26), SSC Register (S27), Engineering Schedule &amp; V&amp;V Report for safety controls (S28) and Design Substantiation Report (S29) removed in Stages 1 to 5, including Plan Safe's share of S28 and S29. Value = their price in the original offer (offer hours × offer sell rates) in those stages."</f>
-        <v>SSC Categorisation Report (S26), SSC Register (S27), Engineering Schedule &amp; V&amp;V Report for safety controls (S28) and Design Substantiation Report (S29) removed in Stages 1 to 5, including Plan Safe's share of S28 and S29. Value = their price in the original offer (offer hours × offer sell rates) in those stages.</v>
+        <f aca="false">"SSC Categorisation Report (S26), SSC Register (S27), Engineering Schedule &amp; V&amp;V Report for safety controls (S28) and Design Substantiation Report (S29) removed in all stages (1 to 7), including Plan Safe's share of S28 and S29. Value = their price in the original offer (offer hours × offer sell rates)."</f>
+        <v>SSC Categorisation Report (S26), SSC Register (S27), Engineering Schedule &amp; V&amp;V Report for safety controls (S28) and Design Substantiation Report (S29) removed in all stages (1 to 7), including Plan Safe's share of S28 and S29. Value = their price in the original offer (offer hours × offer sell rates).</v>
       </c>
       <c r="F4" s="7" t="s">
         <v>16</v>
@@ -862,7 +859,7 @@
         <v>18</v>
       </c>
       <c r="D5" s="5" t="n">
-        <v>167901.940377778</v>
+        <v>152716.325877778</v>
       </c>
       <c r="E5" s="6" t="s">
         <v>19</v>
@@ -951,33 +948,33 @@
         <v>27</v>
       </c>
       <c r="G8" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="H8" s="7" t="s">
         <v>28</v>
-      </c>
-      <c r="H8" s="7" t="s">
-        <v>29</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B9" s="7" t="n">
         <v>7</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="D9" s="9"/>
       <c r="E9" s="8"/>
       <c r="F9" s="8"/>
       <c r="G9" s="8"/>
       <c r="H9" s="7" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B10" s="7" t="n">
         <v>8</v>
@@ -988,12 +985,12 @@
       <c r="F10" s="8"/>
       <c r="G10" s="8"/>
       <c r="H10" s="7" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B11" s="7" t="n">
         <v>9</v>
@@ -1004,12 +1001,12 @@
       <c r="F11" s="8"/>
       <c r="G11" s="8"/>
       <c r="H11" s="7" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B12" s="7" t="n">
         <v>10</v>
@@ -1020,12 +1017,12 @@
       <c r="F12" s="8"/>
       <c r="G12" s="8"/>
       <c r="H12" s="7" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="B13" s="7" t="n">
         <v>11</v>
@@ -1036,30 +1033,30 @@
       <c r="F13" s="8"/>
       <c r="G13" s="8"/>
       <c r="H13" s="7" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C15" s="10" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D15" s="11" t="n">
         <f aca="false">SUM(D3:D7)</f>
-        <v>1923336.02843333</v>
+        <v>2309816.88893333</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C16" s="10" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D16" s="11" t="n">
         <f aca="false">SUM(D3:D8)</f>
-        <v>3145051.55843333</v>
+        <v>3531532.41893333</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C17" s="10" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D17" s="11" t="n">
         <f aca="false">SUM(D9:D13)</f>
@@ -1068,12 +1065,12 @@
     </row>
     <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
   </sheetData>
@@ -1105,7 +1102,7 @@
   <sheetData>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="12" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B2" s="12"/>
       <c r="C2" s="12"/>
@@ -1118,31 +1115,31 @@
     </row>
     <row r="3" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="B3" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="C3" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="D3" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="E3" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="F3" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="F3" s="3" t="s">
+      <c r="G3" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="G3" s="3" t="s">
+      <c r="H3" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="H3" s="3" t="s">
+      <c r="I3" s="3" t="s">
         <v>46</v>
-      </c>
-      <c r="I3" s="3" t="s">
-        <v>47</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1153,29 +1150,29 @@
         <v>335082.825</v>
       </c>
       <c r="C4" s="15" t="n">
-        <v>229226.532693237</v>
+        <v>229164.869624349</v>
       </c>
       <c r="D4" s="15" t="n">
-        <v>121159.482693237</v>
+        <v>121097.819624349</v>
       </c>
       <c r="E4" s="14" t="n">
         <v>106000</v>
       </c>
       <c r="F4" s="16" t="n">
         <f aca="false">IF(B4=0,0,1-C4/B4)</f>
-        <v>0.315910826843372</v>
+        <v>0.316094850208008</v>
       </c>
       <c r="G4" s="16" t="n">
         <f aca="false">IF(B4=0,0,1-D4/B4)</f>
-        <v>0.638419299188978</v>
+        <v>0.638603322553613</v>
       </c>
       <c r="H4" s="17" t="n">
         <f aca="false">IF(C4=0,0,(E4-C4)/C4)</f>
-        <v>-0.537575346297914</v>
+        <v>-0.537450918311533</v>
       </c>
       <c r="I4" s="17" t="n">
         <f aca="false">IF(D4=0,0,(E4-D4)/D4)</f>
-        <v>-0.125120067833396</v>
+        <v>-0.12467457854471</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1186,199 +1183,199 @@
         <v>732839.1</v>
       </c>
       <c r="C5" s="15" t="n">
-        <v>294474.780970431</v>
+        <v>294268.667883964</v>
       </c>
       <c r="D5" s="15" t="n">
-        <v>135608.205970431</v>
+        <v>135402.092883964</v>
       </c>
       <c r="E5" s="14" t="n">
         <v>453000</v>
       </c>
       <c r="F5" s="16" t="n">
         <f aca="false">IF(B5=0,0,1-C5/B5)</f>
-        <v>0.598172667137396</v>
+        <v>0.598453919988762</v>
       </c>
       <c r="G5" s="16" t="n">
         <f aca="false">IF(B5=0,0,1-D5/B5)</f>
-        <v>0.814955007217231</v>
+        <v>0.815236260068596</v>
       </c>
       <c r="H5" s="17" t="n">
         <f aca="false">IF(C5=0,0,(E5-C5)/C5)</f>
-        <v>0.53833207212908</v>
+        <v>0.539409558134225</v>
       </c>
       <c r="I5" s="17" t="n">
         <f aca="false">IF(D5=0,0,(E5-D5)/D5)</f>
-        <v>2.34050581053167</v>
+        <v>2.34559082767065</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B6" s="14" t="n">
         <v>1469323.8</v>
       </c>
       <c r="C6" s="15" t="n">
-        <v>1138296.28283098</v>
+        <v>1136847.12664142</v>
       </c>
       <c r="D6" s="15" t="n">
-        <v>948489.882830978</v>
+        <v>947040.72664142</v>
       </c>
       <c r="E6" s="14" t="n">
         <v>1250000</v>
       </c>
       <c r="F6" s="16" t="n">
         <f aca="false">IF(B6=0,0,1-C6/B6)</f>
-        <v>0.225292421703793</v>
+        <v>0.226278695927052</v>
       </c>
       <c r="G6" s="16" t="n">
         <f aca="false">IF(B6=0,0,1-D6/B6)</f>
-        <v>0.35447184423816</v>
+        <v>0.355458118461417</v>
       </c>
       <c r="H6" s="17" t="n">
         <f aca="false">IF(C6=0,0,(E6-C6)/C6)</f>
-        <v>0.0981323745441822</v>
+        <v>0.0995321804549631</v>
       </c>
       <c r="I6" s="17" t="n">
         <f aca="false">IF(D6=0,0,(E6-D6)/D6)</f>
-        <v>0.317884378765431</v>
+        <v>0.319900997745887</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B7" s="14" t="n">
         <v>3183882.555</v>
       </c>
       <c r="C7" s="15" t="n">
-        <v>2447168.9820988</v>
+        <v>2444083.52602817</v>
       </c>
       <c r="D7" s="15" t="n">
-        <v>2014064.3520988</v>
+        <v>2010978.89602817</v>
       </c>
       <c r="E7" s="14" t="n">
         <v>1455000</v>
       </c>
       <c r="F7" s="16" t="n">
         <f aca="false">IF(B7=0,0,1-C7/B7)</f>
-        <v>0.231388425978294</v>
+        <v>0.232357511997433</v>
       </c>
       <c r="G7" s="16" t="n">
         <f aca="false">IF(B7=0,0,1-D7/B7)</f>
-        <v>0.367418767084893</v>
+        <v>0.368387853104032</v>
       </c>
       <c r="H7" s="17" t="n">
         <f aca="false">IF(C7=0,0,(E7-C7)/C7)</f>
-        <v>-0.405435419195234</v>
+        <v>-0.404684829914757</v>
       </c>
       <c r="I7" s="17" t="n">
         <f aca="false">IF(D7=0,0,(E7-D7)/D7)</f>
-        <v>-0.277580183332382</v>
+        <v>-0.276471770602003</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="13" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B8" s="14" t="n">
         <v>540610.875</v>
       </c>
       <c r="C8" s="15" t="n">
-        <v>284773.170543182</v>
+        <v>284545.536548016</v>
       </c>
       <c r="D8" s="15" t="n">
-        <v>156240.045543182</v>
+        <v>156012.411548016</v>
       </c>
       <c r="E8" s="14" t="n">
         <v>370000</v>
       </c>
       <c r="F8" s="16" t="n">
         <f aca="false">IF(B8=0,0,1-C8/B8)</f>
-        <v>0.473238176085189</v>
+        <v>0.473659244187391</v>
       </c>
       <c r="G8" s="16" t="n">
         <f aca="false">IF(B8=0,0,1-D8/B8)</f>
-        <v>0.710993520906915</v>
+        <v>0.711414589009117</v>
       </c>
       <c r="H8" s="17" t="n">
         <f aca="false">IF(C8=0,0,(E8-C8)/C8)</f>
-        <v>0.299279701434846</v>
+        <v>0.300319114081636</v>
       </c>
       <c r="I8" s="17" t="n">
         <f aca="false">IF(D8=0,0,(E8-D8)/D8)</f>
-        <v>1.36815087139576</v>
+        <v>1.37160618394854</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="13" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B9" s="14" t="n">
         <v>775079.55</v>
       </c>
       <c r="C9" s="15" t="n">
-        <v>742522.76735156</v>
+        <v>490533.729962928</v>
       </c>
       <c r="D9" s="15" t="n">
-        <v>595633.01735156</v>
+        <v>343643.979962928</v>
       </c>
       <c r="E9" s="14" t="n">
         <v>102000</v>
       </c>
       <c r="F9" s="16" t="n">
         <f aca="false">IF(B9=0,0,1-C9/B9)</f>
-        <v>0.0420044402518943</v>
+        <v>0.367118213913749</v>
       </c>
       <c r="G9" s="16" t="n">
         <f aca="false">IF(B9=0,0,1-D9/B9)</f>
-        <v>0.231520148671759</v>
+        <v>0.556633922333613</v>
       </c>
       <c r="H9" s="17" t="n">
         <f aca="false">IF(C9=0,0,(E9-C9)/C9)</f>
-        <v>-0.862630474801716</v>
+        <v>-0.792063228745333</v>
       </c>
       <c r="I9" s="17" t="n">
         <f aca="false">IF(D9=0,0,(E9-D9)/D9)</f>
-        <v>-0.82875361669248</v>
+        <v>-0.703181181841149</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="13" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B10" s="14" t="n">
         <v>493905.3</v>
       </c>
       <c r="C10" s="15" t="n">
-        <v>470925.460078476</v>
+        <v>341463.659377819</v>
       </c>
       <c r="D10" s="15" t="n">
-        <v>414477.460078476</v>
+        <v>285015.659377819</v>
       </c>
       <c r="E10" s="14" t="n">
         <v>73000</v>
       </c>
       <c r="F10" s="16" t="n">
         <f aca="false">IF(B10=0,0,1-C10/B10)</f>
-        <v>0.0465268137870235</v>
+        <v>0.308645484513288</v>
       </c>
       <c r="G10" s="16" t="n">
         <f aca="false">IF(B10=0,0,1-D10/B10)</f>
-        <v>0.160815929534516</v>
+        <v>0.422934600260781</v>
       </c>
       <c r="H10" s="17" t="n">
         <f aca="false">IF(C10=0,0,(E10-C10)/C10)</f>
-        <v>-0.844986083386031</v>
+        <v>-0.786214438944943</v>
       </c>
       <c r="I10" s="17" t="n">
         <f aca="false">IF(D10=0,0,(E10-D10)/D10)</f>
-        <v>-0.823874620380615</v>
+        <v>-0.743873722028618</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="18" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B11" s="19" t="n">
         <f aca="false">SUM(B4:B10)</f>
@@ -1386,11 +1383,11 @@
       </c>
       <c r="C11" s="19" t="n">
         <f aca="false">SUM(C4:C10)</f>
-        <v>5607387.97656667</v>
+        <v>5220907.11606667</v>
       </c>
       <c r="D11" s="19" t="n">
         <f aca="false">SUM(D4:D10)</f>
-        <v>4385672.44656666</v>
+        <v>3999191.58606667</v>
       </c>
       <c r="E11" s="19" t="n">
         <f aca="false">SUM(E4:E10)</f>
@@ -1398,19 +1395,19 @@
       </c>
       <c r="F11" s="20" t="n">
         <f aca="false">IF(B11=0,0,1-C11/B11)</f>
-        <v>0.255398554927301</v>
+        <v>0.306719099969636</v>
       </c>
       <c r="G11" s="20" t="n">
         <f aca="false">IF(B11=0,0,1-D11/B11)</f>
-        <v>0.417629374857609</v>
+        <v>0.468949919899944</v>
       </c>
       <c r="H11" s="21" t="n">
         <f aca="false">IF(C11=0,0,(E11-C11)/C11)</f>
-        <v>-0.320717593304075</v>
+        <v>-0.2704332953409</v>
       </c>
       <c r="I11" s="21" t="n">
         <f aca="false">IF(D11=0,0,(E11-D11)/D11)</f>
-        <v>-0.131490085863141</v>
+        <v>-0.047557508054703</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1418,7 +1415,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="12" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12"/>
@@ -1431,25 +1428,25 @@
     </row>
     <row r="14" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="B14" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="B14" s="3" t="s">
-        <v>40</v>
-      </c>
       <c r="C14" s="3" t="s">
+        <v>54</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>31</v>
+      </c>
+      <c r="E14" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="D14" s="3" t="s">
-        <v>32</v>
-      </c>
-      <c r="E14" s="3" t="s">
+      <c r="F14" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="F14" s="3" t="s">
+      <c r="G14" s="3" t="s">
         <v>57</v>
-      </c>
-      <c r="G14" s="3" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1494,7 +1491,7 @@
     </row>
     <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="13" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B17" s="23"/>
       <c r="C17" s="23"/>
@@ -1514,7 +1511,7 @@
     </row>
     <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="13" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B18" s="23"/>
       <c r="C18" s="23"/>
@@ -1534,7 +1531,7 @@
     </row>
     <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="13" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B19" s="23"/>
       <c r="C19" s="23"/>
@@ -1554,7 +1551,7 @@
     </row>
     <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="13" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B20" s="23"/>
       <c r="C20" s="23"/>
@@ -1574,7 +1571,7 @@
     </row>
     <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="13" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B21" s="23"/>
       <c r="C21" s="23"/>
@@ -1594,7 +1591,7 @@
     </row>
     <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="18" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B22" s="19" t="n">
         <f aca="false">SUM(B15:B21)</f>
@@ -1629,12 +1626,12 @@
     </row>
     <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="2" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="12" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B26" s="12"/>
       <c r="C26" s="12"/>
@@ -1647,31 +1644,31 @@
     </row>
     <row r="27" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="3" t="s">
+        <v>38</v>
+      </c>
+      <c r="B27" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="B27" s="3" t="s">
-        <v>40</v>
-      </c>
       <c r="C27" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="D27" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="D27" s="3" t="s">
+      <c r="E27" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="E27" s="3" t="s">
+      <c r="F27" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="G27" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="H27" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="F27" s="3" t="s">
-        <v>44</v>
-      </c>
-      <c r="G27" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="H27" s="3" t="s">
+      <c r="I27" s="3" t="s">
         <v>64</v>
-      </c>
-      <c r="I27" s="3" t="s">
-        <v>65</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1684,11 +1681,11 @@
       </c>
       <c r="C28" s="15" t="n">
         <f aca="false">C4+D15</f>
-        <v>229226.532693237</v>
+        <v>229164.869624349</v>
       </c>
       <c r="D28" s="15" t="n">
         <f aca="false">D4+D15</f>
-        <v>121159.482693237</v>
+        <v>121097.819624349</v>
       </c>
       <c r="E28" s="14" t="n">
         <f aca="false">E4+N(E15)</f>
@@ -1696,19 +1693,19 @@
       </c>
       <c r="F28" s="16" t="n">
         <f aca="false">IF(B28=0,0,1-C28/B28)</f>
-        <v>0.315910826843372</v>
+        <v>0.316094850208008</v>
       </c>
       <c r="G28" s="16" t="n">
         <f aca="false">IF(B28=0,0,1-D28/B28)</f>
-        <v>0.638419299188978</v>
+        <v>0.638603322553613</v>
       </c>
       <c r="H28" s="17" t="n">
         <f aca="false">IF(C28=0,0,(E28-C28)/C28)</f>
-        <v>-0.537575346297914</v>
+        <v>-0.537450918311533</v>
       </c>
       <c r="I28" s="17" t="n">
         <f aca="false">IF(D28=0,0,(E28-D28)/D28)</f>
-        <v>-0.125120067833396</v>
+        <v>-0.12467457854471</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1721,11 +1718,11 @@
       </c>
       <c r="C29" s="15" t="n">
         <f aca="false">C5+D16</f>
-        <v>294474.780970431</v>
+        <v>294268.667883964</v>
       </c>
       <c r="D29" s="15" t="n">
         <f aca="false">D5+D16</f>
-        <v>135608.205970431</v>
+        <v>135402.092883964</v>
       </c>
       <c r="E29" s="14" t="n">
         <f aca="false">E5+N(E16)</f>
@@ -1733,24 +1730,24 @@
       </c>
       <c r="F29" s="16" t="n">
         <f aca="false">IF(B29=0,0,1-C29/B29)</f>
-        <v>0.598172667137396</v>
+        <v>0.598453919988762</v>
       </c>
       <c r="G29" s="16" t="n">
         <f aca="false">IF(B29=0,0,1-D29/B29)</f>
-        <v>0.814955007217231</v>
+        <v>0.815236260068596</v>
       </c>
       <c r="H29" s="17" t="n">
         <f aca="false">IF(C29=0,0,(E29-C29)/C29)</f>
-        <v>0.53833207212908</v>
+        <v>0.539409558134225</v>
       </c>
       <c r="I29" s="17" t="n">
         <f aca="false">IF(D29=0,0,(E29-D29)/D29)</f>
-        <v>2.34050581053167</v>
+        <v>2.34559082767065</v>
       </c>
     </row>
     <row r="30" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="13" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B30" s="14" t="n">
         <f aca="false">B6+N(B17)</f>
@@ -1758,11 +1755,11 @@
       </c>
       <c r="C30" s="15" t="n">
         <f aca="false">C6+D17</f>
-        <v>1138296.28283098</v>
+        <v>1136847.12664142</v>
       </c>
       <c r="D30" s="15" t="n">
         <f aca="false">D6+D17</f>
-        <v>948489.882830978</v>
+        <v>947040.72664142</v>
       </c>
       <c r="E30" s="14" t="n">
         <f aca="false">E6+N(E17)</f>
@@ -1770,24 +1767,24 @@
       </c>
       <c r="F30" s="16" t="n">
         <f aca="false">IF(B30=0,0,1-C30/B30)</f>
-        <v>0.225292421703793</v>
+        <v>0.226278695927052</v>
       </c>
       <c r="G30" s="16" t="n">
         <f aca="false">IF(B30=0,0,1-D30/B30)</f>
-        <v>0.35447184423816</v>
+        <v>0.355458118461417</v>
       </c>
       <c r="H30" s="17" t="n">
         <f aca="false">IF(C30=0,0,(E30-C30)/C30)</f>
-        <v>0.0981323745441822</v>
+        <v>0.0995321804549631</v>
       </c>
       <c r="I30" s="17" t="n">
         <f aca="false">IF(D30=0,0,(E30-D30)/D30)</f>
-        <v>0.317884378765431</v>
+        <v>0.319900997745887</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="13" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B31" s="14" t="n">
         <f aca="false">B7+N(B18)</f>
@@ -1795,11 +1792,11 @@
       </c>
       <c r="C31" s="15" t="n">
         <f aca="false">C7+D18</f>
-        <v>2447168.9820988</v>
+        <v>2444083.52602817</v>
       </c>
       <c r="D31" s="15" t="n">
         <f aca="false">D7+D18</f>
-        <v>2014064.3520988</v>
+        <v>2010978.89602817</v>
       </c>
       <c r="E31" s="14" t="n">
         <f aca="false">E7+N(E18)</f>
@@ -1807,24 +1804,24 @@
       </c>
       <c r="F31" s="16" t="n">
         <f aca="false">IF(B31=0,0,1-C31/B31)</f>
-        <v>0.231388425978294</v>
+        <v>0.232357511997433</v>
       </c>
       <c r="G31" s="16" t="n">
         <f aca="false">IF(B31=0,0,1-D31/B31)</f>
-        <v>0.367418767084893</v>
+        <v>0.368387853104032</v>
       </c>
       <c r="H31" s="17" t="n">
         <f aca="false">IF(C31=0,0,(E31-C31)/C31)</f>
-        <v>-0.405435419195234</v>
+        <v>-0.404684829914757</v>
       </c>
       <c r="I31" s="17" t="n">
         <f aca="false">IF(D31=0,0,(E31-D31)/D31)</f>
-        <v>-0.277580183332382</v>
+        <v>-0.276471770602003</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="13" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B32" s="14" t="n">
         <f aca="false">B8+N(B19)</f>
@@ -1832,11 +1829,11 @@
       </c>
       <c r="C32" s="15" t="n">
         <f aca="false">C8+D19</f>
-        <v>284773.170543182</v>
+        <v>284545.536548016</v>
       </c>
       <c r="D32" s="15" t="n">
         <f aca="false">D8+D19</f>
-        <v>156240.045543182</v>
+        <v>156012.411548016</v>
       </c>
       <c r="E32" s="14" t="n">
         <f aca="false">E8+N(E19)</f>
@@ -1844,24 +1841,24 @@
       </c>
       <c r="F32" s="16" t="n">
         <f aca="false">IF(B32=0,0,1-C32/B32)</f>
-        <v>0.473238176085189</v>
+        <v>0.473659244187391</v>
       </c>
       <c r="G32" s="16" t="n">
         <f aca="false">IF(B32=0,0,1-D32/B32)</f>
-        <v>0.710993520906915</v>
+        <v>0.711414589009117</v>
       </c>
       <c r="H32" s="17" t="n">
         <f aca="false">IF(C32=0,0,(E32-C32)/C32)</f>
-        <v>0.299279701434846</v>
+        <v>0.300319114081636</v>
       </c>
       <c r="I32" s="17" t="n">
         <f aca="false">IF(D32=0,0,(E32-D32)/D32)</f>
-        <v>1.36815087139576</v>
+        <v>1.37160618394854</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="13" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B33" s="14" t="n">
         <f aca="false">B9+N(B20)</f>
@@ -1869,11 +1866,11 @@
       </c>
       <c r="C33" s="15" t="n">
         <f aca="false">C9+D20</f>
-        <v>742522.76735156</v>
+        <v>490533.729962928</v>
       </c>
       <c r="D33" s="15" t="n">
         <f aca="false">D9+D20</f>
-        <v>595633.01735156</v>
+        <v>343643.979962928</v>
       </c>
       <c r="E33" s="14" t="n">
         <f aca="false">E9+N(E20)</f>
@@ -1881,24 +1878,24 @@
       </c>
       <c r="F33" s="16" t="n">
         <f aca="false">IF(B33=0,0,1-C33/B33)</f>
-        <v>0.0420044402518943</v>
+        <v>0.367118213913749</v>
       </c>
       <c r="G33" s="16" t="n">
         <f aca="false">IF(B33=0,0,1-D33/B33)</f>
-        <v>0.231520148671759</v>
+        <v>0.556633922333613</v>
       </c>
       <c r="H33" s="17" t="n">
         <f aca="false">IF(C33=0,0,(E33-C33)/C33)</f>
-        <v>-0.862630474801716</v>
+        <v>-0.792063228745333</v>
       </c>
       <c r="I33" s="17" t="n">
         <f aca="false">IF(D33=0,0,(E33-D33)/D33)</f>
-        <v>-0.82875361669248</v>
+        <v>-0.703181181841149</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="13" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B34" s="14" t="n">
         <f aca="false">B10+N(B21)</f>
@@ -1906,11 +1903,11 @@
       </c>
       <c r="C34" s="15" t="n">
         <f aca="false">C10+D21</f>
-        <v>470925.460078476</v>
+        <v>341463.659377819</v>
       </c>
       <c r="D34" s="15" t="n">
         <f aca="false">D10+D21</f>
-        <v>414477.460078476</v>
+        <v>285015.659377819</v>
       </c>
       <c r="E34" s="14" t="n">
         <f aca="false">E10+N(E21)</f>
@@ -1918,24 +1915,24 @@
       </c>
       <c r="F34" s="16" t="n">
         <f aca="false">IF(B34=0,0,1-C34/B34)</f>
-        <v>0.0465268137870235</v>
+        <v>0.308645484513288</v>
       </c>
       <c r="G34" s="16" t="n">
         <f aca="false">IF(B34=0,0,1-D34/B34)</f>
-        <v>0.160815929534516</v>
+        <v>0.422934600260781</v>
       </c>
       <c r="H34" s="17" t="n">
         <f aca="false">IF(C34=0,0,(E34-C34)/C34)</f>
-        <v>-0.844986083386031</v>
+        <v>-0.786214438944943</v>
       </c>
       <c r="I34" s="17" t="n">
         <f aca="false">IF(D34=0,0,(E34-D34)/D34)</f>
-        <v>-0.823874620380615</v>
+        <v>-0.743873722028618</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="18" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B35" s="19" t="n">
         <f aca="false">SUM(B28:B34)</f>
@@ -1943,11 +1940,11 @@
       </c>
       <c r="C35" s="19" t="n">
         <f aca="false">SUM(C28:C34)</f>
-        <v>5607387.97656667</v>
+        <v>5220907.11606667</v>
       </c>
       <c r="D35" s="19" t="n">
         <f aca="false">SUM(D28:D34)</f>
-        <v>4385672.44656666</v>
+        <v>3999191.58606667</v>
       </c>
       <c r="E35" s="19" t="n">
         <f aca="false">SUM(E28:E34)</f>
@@ -1955,24 +1952,24 @@
       </c>
       <c r="F35" s="20" t="n">
         <f aca="false">IF(B35=0,0,1-C35/B35)</f>
-        <v>0.255398554927301</v>
+        <v>0.306719099969636</v>
       </c>
       <c r="G35" s="20" t="n">
         <f aca="false">IF(B35=0,0,1-D35/B35)</f>
-        <v>0.417629374857609</v>
+        <v>0.468949919899944</v>
       </c>
       <c r="H35" s="21" t="n">
         <f aca="false">IF(C35=0,0,(E35-C35)/C35)</f>
-        <v>-0.320717593304075</v>
+        <v>-0.2704332953409</v>
       </c>
       <c r="I35" s="21" t="n">
         <f aca="false">IF(D35=0,0,(E35-D35)/D35)</f>
-        <v>-0.131490085863141</v>
+        <v>-0.047557508054703</v>
       </c>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="12" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B38" s="12"/>
       <c r="C38" s="12"/>
@@ -1985,44 +1982,44 @@
     </row>
     <row r="39" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="B39" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="C39" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="D39" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="E39" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="B39" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="C39" s="3" t="s">
-        <v>41</v>
-      </c>
-      <c r="D39" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="E39" s="3" t="s">
+      <c r="F39" s="3" t="s">
         <v>68</v>
-      </c>
-      <c r="F39" s="3" t="s">
-        <v>69</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="24" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B40" s="14" t="n">
         <v>5858217.9075</v>
       </c>
       <c r="C40" s="14" t="n">
-        <v>4029646.56906667</v>
+        <v>3665191.82106667</v>
       </c>
       <c r="D40" s="14" t="n">
-        <v>4029646.56906667</v>
+        <v>3665191.82106667</v>
       </c>
       <c r="E40" s="14" t="n">
         <f aca="false">B40-C40</f>
-        <v>1828571.33843333</v>
+        <v>2193026.08643333</v>
       </c>
       <c r="F40" s="14" t="n">
         <f aca="false">B40-D40</f>
-        <v>1828571.33843333</v>
+        <v>2193026.08643333</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2033,23 +2030,23 @@
         <v>1593669.9975</v>
       </c>
       <c r="C41" s="14" t="n">
-        <v>1498905.3075</v>
+        <v>1476879.195</v>
       </c>
       <c r="D41" s="14" t="n">
-        <v>277189.7775</v>
+        <v>255163.665</v>
       </c>
       <c r="E41" s="14" t="n">
         <f aca="false">B41-C41</f>
-        <v>94764.6899999999</v>
+        <v>116790.8025</v>
       </c>
       <c r="F41" s="14" t="n">
         <f aca="false">B41-D41</f>
-        <v>1316480.22</v>
+        <v>1338506.3325</v>
       </c>
     </row>
     <row r="42" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="24" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B42" s="14" t="n">
         <v>78836.1</v>
@@ -2071,7 +2068,7 @@
     </row>
     <row r="43" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="10" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B43" s="19" t="n">
         <f aca="false">SUM(B40:B42)</f>
@@ -2079,24 +2076,24 @@
       </c>
       <c r="C43" s="19" t="n">
         <f aca="false">SUM(C40:C42)</f>
-        <v>5607387.97656667</v>
+        <v>5220907.11606667</v>
       </c>
       <c r="D43" s="19" t="n">
         <f aca="false">SUM(D40:D42)</f>
-        <v>4385672.44656667</v>
+        <v>3999191.58606667</v>
       </c>
       <c r="E43" s="19" t="n">
         <f aca="false">SUM(E40:E42)</f>
-        <v>1923336.02843333</v>
+        <v>2309816.88893333</v>
       </c>
       <c r="F43" s="19" t="n">
         <f aca="false">SUM(F40:F42)</f>
-        <v>3145051.55843333</v>
+        <v>3531532.41893333</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="2" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Use the agreed justifications for rework, SSC scope and management overlap adjustment
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016KmKbhNhfEuuXeBfiH8ZpM
</commit_message>
<xml_diff>
--- a/NMMP_Reductions_Nuclear_Pharma.xlsx
+++ b/NMMP_Reductions_Nuclear_Pharma.xlsx
@@ -21,9 +21,9 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="72">
-  <si>
-    <t xml:space="preserve">Reductions on the NMMP offer — all amounts in AUD. Nuclear reductions are applied in sequence, without double counting: SSC descoping → S1 deliverable adjustment → rework → travel → commercial discount. Plan Safe applies to Scenario 2 only.</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="73">
+  <si>
+    <t xml:space="preserve">Reductions on the NMMP offer — all amounts in AUD. Nuclear reductions are applied in sequence, without double counting: SSC descoping → S1 deliverable adjustment → rework → travel → management overlap adjustment (4%). Plan Safe applies to Scenario 2 only.</t>
   </si>
   <si>
     <t xml:space="preserve">Discipline</t>
@@ -53,10 +53,10 @@
     <t xml:space="preserve">Nuclear</t>
   </si>
   <si>
-    <t xml:space="preserve">Rework</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The 35% rework allowance on IDOM's Stage 2 tasks is released in full: all deliverables are assumed right first time. Calculated on IDOM's Stage 2 amount remaining after the SSC descoping and the S1 deliverable adjustment (180,964 AUD × 35/135). On the original offer it would be 139,097 AUD.</t>
+    <t xml:space="preserve">Rework allowance</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The original estimate included a specific allowance for potential rework during Concept Design, reflecting the risk associated with the completeness, accuracy and maturity of the design information and inputs available at tender stage. For the revised commercial position, this allowance has been removed on the basis that the information provided to IDOM will be complete, accurate and sufficiently mature to perform the agreed scope without redesign or rework of previously completed activities. Any material change, correction, late information or insufficient input requiring rework of completed activities will be treated as a change to the agreed scope and subject to prior agreement on the corresponding programme and commercial impact.</t>
   </si>
   <si>
     <t xml:space="preserve">n/a</t>
@@ -68,7 +68,10 @@
     <t xml:space="preserve">Scenarios 1 and 2</t>
   </si>
   <si>
-    <t xml:space="preserve">SSC descoping</t>
+    <t xml:space="preserve">SSC / Systems Engineering Scope (S26–S29)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">During the scope alignment discussions, Systems Engineering was identified by Synertec as an area of potential overlap between the parties. To eliminate duplication and establish clear accountability, IDOM is prepared to remove the full S26–S29 scope from its offer. These deliverables relate to facility-wide SSC categorisation, register management, safety controls V&amp;V and design substantiation, and are closely linked to the overall design integration and systems engineering activities performed across the PDDI. Consolidating ownership of this scope under Synertec therefore provides a clearer and more efficient interface model. Accordingly, S26–S29 will be transferred to Synertec’s scope.</t>
   </si>
   <si>
     <t xml:space="preserve">S26, S27, S28, S29</t>
@@ -77,10 +80,10 @@
     <t xml:space="preserve">S1-S7</t>
   </si>
   <si>
-    <t xml:space="preserve">Commercial discount</t>
-  </si>
-  <si>
-    <t xml:space="preserve">4% discount on everything IDOM invoices, applied after the other reductions (3,817,908 AUD × 4%). Not applied to Plan Safe or INVAP.</t>
+    <t xml:space="preserve">Management Overlap Adjustment – 4%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Following receipt of Synertec’s organisational structure, IDOM identified potential overlap in certain management roles that was not visible at the time of the original submission. Based on this improved understanding of the proposed delivery model, IDOM has reviewed the management-related effort and is able to apply a 4% reduction to the Nuclear &amp; Radiological scope, reflecting the removal of potential duplicated management effort and improved alignment between the parties. The underlying technical scope remains unchanged.</t>
   </si>
   <si>
     <t xml:space="preserve">All</t>
@@ -795,7 +798,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="150" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
         <v>9</v>
       </c>
@@ -821,7 +824,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="135" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
         <v>9</v>
       </c>
@@ -834,21 +837,20 @@
       <c r="D4" s="5" t="n">
         <v>1652324.1</v>
       </c>
-      <c r="E4" s="6" t="str">
-        <f aca="false">"SSC Categorisation Report (S26), SSC Register (S27), Engineering Schedule &amp; V&amp;V Report for safety controls (S28) and Design Substantiation Report (S29) removed in all stages (1 to 7), including Plan Safe's share of S28 and S29. Value = their price in the original offer (offer hours × offer sell rates)."</f>
-        <v>SSC Categorisation Report (S26), SSC Register (S27), Engineering Schedule &amp; V&amp;V Report for safety controls (S28) and Design Substantiation Report (S29) removed in all stages (1 to 7), including Plan Safe's share of S28 and S29. Value = their price in the original offer (offer hours × offer sell rates).</v>
+      <c r="E4" s="6" t="s">
+        <v>16</v>
       </c>
       <c r="F4" s="7" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="G4" s="7" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="H4" s="7" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="135" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
         <v>9</v>
       </c>
@@ -856,19 +858,19 @@
         <v>3</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D5" s="5" t="n">
         <v>152716.325877778</v>
       </c>
       <c r="E5" s="6" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F5" s="7" t="s">
         <v>12</v>
       </c>
       <c r="G5" s="7" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="H5" s="7" t="s">
         <v>14</v>
@@ -882,19 +884,19 @@
         <v>4</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D6" s="5" t="n">
         <v>387859.875</v>
       </c>
       <c r="E6" s="6" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="F6" s="7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G6" s="7" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="H6" s="7" t="s">
         <v>14</v>
@@ -908,7 +910,7 @@
         <v>5</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="D7" s="5" t="n">
         <v>70000</v>
@@ -921,7 +923,7 @@
         <v>12</v>
       </c>
       <c r="G7" s="7" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="H7" s="7" t="s">
         <v>14</v>
@@ -935,7 +937,7 @@
         <v>6</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D8" s="5" t="n">
         <v>1221715.53</v>
@@ -945,36 +947,36 @@
         <v>Plan Safe's own human factors deliverables removed (HF Assurance / Integration Plan, HF Hazards Identification and Control Plan, HF Task Assessments, HF Substantiation Report). Value = their price in the original offer. Plan Safe keeps its share of the shared deliverables.</v>
       </c>
       <c r="F8" s="7" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="G8" s="7" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="H8" s="7" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B9" s="7" t="n">
         <v>7</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D9" s="9"/>
       <c r="E9" s="8"/>
       <c r="F9" s="8"/>
       <c r="G9" s="8"/>
       <c r="H9" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B10" s="7" t="n">
         <v>8</v>
@@ -985,12 +987,12 @@
       <c r="F10" s="8"/>
       <c r="G10" s="8"/>
       <c r="H10" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B11" s="7" t="n">
         <v>9</v>
@@ -1001,12 +1003,12 @@
       <c r="F11" s="8"/>
       <c r="G11" s="8"/>
       <c r="H11" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B12" s="7" t="n">
         <v>10</v>
@@ -1017,12 +1019,12 @@
       <c r="F12" s="8"/>
       <c r="G12" s="8"/>
       <c r="H12" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B13" s="7" t="n">
         <v>11</v>
@@ -1033,12 +1035,12 @@
       <c r="F13" s="8"/>
       <c r="G13" s="8"/>
       <c r="H13" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C15" s="10" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D15" s="11" t="n">
         <f aca="false">SUM(D3:D7)</f>
@@ -1047,7 +1049,7 @@
     </row>
     <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C16" s="10" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D16" s="11" t="n">
         <f aca="false">SUM(D3:D8)</f>
@@ -1056,7 +1058,7 @@
     </row>
     <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C17" s="10" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D17" s="11" t="n">
         <f aca="false">SUM(D9:D13)</f>
@@ -1065,12 +1067,12 @@
     </row>
     <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
   </sheetData>
@@ -1102,7 +1104,7 @@
   <sheetData>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="12" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B2" s="12"/>
       <c r="C2" s="12"/>
@@ -1115,36 +1117,36 @@
     </row>
     <row r="3" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="13" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B4" s="14" t="n">
         <v>335082.825</v>
@@ -1210,7 +1212,7 @@
     </row>
     <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B6" s="14" t="n">
         <v>1469323.8</v>
@@ -1243,7 +1245,7 @@
     </row>
     <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B7" s="14" t="n">
         <v>3183882.555</v>
@@ -1276,7 +1278,7 @@
     </row>
     <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="13" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B8" s="14" t="n">
         <v>540610.875</v>
@@ -1309,7 +1311,7 @@
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="13" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B9" s="14" t="n">
         <v>775079.55</v>
@@ -1342,7 +1344,7 @@
     </row>
     <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="13" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B10" s="14" t="n">
         <v>493905.3</v>
@@ -1375,7 +1377,7 @@
     </row>
     <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="18" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B11" s="19" t="n">
         <f aca="false">SUM(B4:B10)</f>
@@ -1415,7 +1417,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="12" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B13" s="12"/>
       <c r="C13" s="12"/>
@@ -1428,30 +1430,30 @@
     </row>
     <row r="14" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="E14" s="3" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="F14" s="3" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="G14" s="3" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="13" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B15" s="23"/>
       <c r="C15" s="23"/>
@@ -1491,7 +1493,7 @@
     </row>
     <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="13" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B17" s="23"/>
       <c r="C17" s="23"/>
@@ -1511,7 +1513,7 @@
     </row>
     <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="13" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B18" s="23"/>
       <c r="C18" s="23"/>
@@ -1531,7 +1533,7 @@
     </row>
     <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="13" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B19" s="23"/>
       <c r="C19" s="23"/>
@@ -1551,7 +1553,7 @@
     </row>
     <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="13" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B20" s="23"/>
       <c r="C20" s="23"/>
@@ -1571,7 +1573,7 @@
     </row>
     <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="13" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B21" s="23"/>
       <c r="C21" s="23"/>
@@ -1591,7 +1593,7 @@
     </row>
     <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="18" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B22" s="19" t="n">
         <f aca="false">SUM(B15:B21)</f>
@@ -1626,12 +1628,12 @@
     </row>
     <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="12" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B26" s="12"/>
       <c r="C26" s="12"/>
@@ -1644,36 +1646,36 @@
     </row>
     <row r="27" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="3" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="D27" s="3" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="E27" s="3" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="F27" s="3" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="G27" s="3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="H27" s="3" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="I27" s="3" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="13" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B28" s="14" t="n">
         <f aca="false">B4+N(B15)</f>
@@ -1747,7 +1749,7 @@
     </row>
     <row r="30" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="13" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B30" s="14" t="n">
         <f aca="false">B6+N(B17)</f>
@@ -1784,7 +1786,7 @@
     </row>
     <row r="31" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="13" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B31" s="14" t="n">
         <f aca="false">B7+N(B18)</f>
@@ -1821,7 +1823,7 @@
     </row>
     <row r="32" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="13" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B32" s="14" t="n">
         <f aca="false">B8+N(B19)</f>
@@ -1858,7 +1860,7 @@
     </row>
     <row r="33" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="13" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B33" s="14" t="n">
         <f aca="false">B9+N(B20)</f>
@@ -1895,7 +1897,7 @@
     </row>
     <row r="34" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="13" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B34" s="14" t="n">
         <f aca="false">B10+N(B21)</f>
@@ -1932,7 +1934,7 @@
     </row>
     <row r="35" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="18" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B35" s="19" t="n">
         <f aca="false">SUM(B28:B34)</f>
@@ -1969,7 +1971,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="12" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="B38" s="12"/>
       <c r="C38" s="12"/>
@@ -1982,27 +1984,27 @@
     </row>
     <row r="39" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="3" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B39" s="3" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C39" s="3" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D39" s="3" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E39" s="3" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F39" s="3" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="24" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B40" s="14" t="n">
         <v>5858217.9075</v>
@@ -2024,7 +2026,7 @@
     </row>
     <row r="41" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="24" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B41" s="14" t="n">
         <v>1593669.9975</v>
@@ -2046,7 +2048,7 @@
     </row>
     <row r="42" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="24" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B42" s="14" t="n">
         <v>78836.1</v>
@@ -2068,7 +2070,7 @@
     </row>
     <row r="43" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="10" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B43" s="19" t="n">
         <f aca="false">SUM(B40:B42)</f>
@@ -2093,7 +2095,7 @@
     </row>
     <row r="45" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="2" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add lump sum S1-S3 and provisional sum S4-S5 / S6-S7 subtotals to the Summary tables
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016KmKbhNhfEuuXeBfiH8ZpM
</commit_message>
<xml_diff>
--- a/NMMP_Reductions_Nuclear_Pharma.xlsx
+++ b/NMMP_Reductions_Nuclear_Pharma.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="76">
   <si>
     <t xml:space="preserve">Reductions on the NMMP offer — all amounts in AUD. Nuclear reductions are applied in sequence, without double counting: SSC descoping → S1 deliverable adjustment → rework → travel → management overlap adjustment (4%). Plan Safe applies to Scenario 2 only.</t>
   </si>
@@ -170,16 +170,25 @@
     <t xml:space="preserve">S3</t>
   </si>
   <si>
+    <t xml:space="preserve">Lump sum S1-S3</t>
+  </si>
+  <si>
     <t xml:space="preserve">S4</t>
   </si>
   <si>
     <t xml:space="preserve">S5</t>
   </si>
   <si>
+    <t xml:space="preserve">Provisional sum S4-S5</t>
+  </si>
+  <si>
     <t xml:space="preserve">S6</t>
   </si>
   <si>
     <t xml:space="preserve">S7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Provisional sum S6-S7</t>
   </si>
   <si>
     <t xml:space="preserve">TOTAL</t>
@@ -331,7 +340,7 @@
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -362,6 +371,12 @@
         <bgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFDDEBF7"/>
+        <bgColor rgb="FFF2F4F7"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border diagonalUp="false" diagonalDown="false">
@@ -404,7 +419,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="28">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -477,8 +492,24 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="10" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+    <xf numFmtId="164" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="166" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
@@ -491,10 +522,6 @@
     </xf>
     <xf numFmtId="168" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="166" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
@@ -535,7 +562,7 @@
       <rgbColor rgb="FF9999FF"/>
       <rgbColor rgb="FF993366"/>
       <rgbColor rgb="FFFFF2CC"/>
-      <rgbColor rgb="FFF2F4F7"/>
+      <rgbColor rgb="FFDDEBF7"/>
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFFF8080"/>
       <rgbColor rgb="FF0070C0"/>
@@ -549,7 +576,7 @@
       <rgbColor rgb="FF008080"/>
       <rgbColor rgb="FF0000FF"/>
       <rgbColor rgb="FF00CCFF"/>
-      <rgbColor rgb="FFCCFFFF"/>
+      <rgbColor rgb="FFF2F4F7"/>
       <rgbColor rgb="FFCCFFCC"/>
       <rgbColor rgb="FFFFFF99"/>
       <rgbColor rgb="FF99CCFF"/>
@@ -798,7 +825,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="150" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="3" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
         <v>9</v>
       </c>
@@ -824,7 +851,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="135" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
         <v>9</v>
       </c>
@@ -850,7 +877,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="135" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="61.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
         <v>9</v>
       </c>
@@ -1091,10 +1118,10 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A2:I45"/>
+  <dimension ref="A2:I54"/>
   <sheetFormatPr defaultColWidth="10.5390625" defaultRowHeight="14.25" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="11"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="14"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="15"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="3" style="1" width="20"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="18"/>
@@ -1243,37 +1270,41 @@
         <v>0.319900997745887</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="13" t="s">
+    <row r="7" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="18" t="s">
         <v>49</v>
       </c>
-      <c r="B7" s="14" t="n">
-        <v>3183882.555</v>
-      </c>
-      <c r="C7" s="15" t="n">
-        <v>2444083.52602817</v>
-      </c>
-      <c r="D7" s="15" t="n">
-        <v>2010978.89602817</v>
-      </c>
-      <c r="E7" s="14" t="n">
-        <v>1455000</v>
-      </c>
-      <c r="F7" s="16" t="n">
+      <c r="B7" s="19" t="n">
+        <f aca="false">N(B4)+N(B5)+N(B6)</f>
+        <v>2537245.725</v>
+      </c>
+      <c r="C7" s="19" t="n">
+        <f aca="false">N(C4)+N(C5)+N(C6)</f>
+        <v>1660280.66414973</v>
+      </c>
+      <c r="D7" s="19" t="n">
+        <f aca="false">N(D4)+N(D5)+N(D6)</f>
+        <v>1203540.63914973</v>
+      </c>
+      <c r="E7" s="19" t="n">
+        <f aca="false">N(E4)+N(E5)+N(E6)</f>
+        <v>1809000</v>
+      </c>
+      <c r="F7" s="20" t="n">
         <f aca="false">IF(B7=0,0,1-C7/B7)</f>
-        <v>0.232357511997433</v>
-      </c>
-      <c r="G7" s="16" t="n">
+        <v>0.345636629597737</v>
+      </c>
+      <c r="G7" s="20" t="n">
         <f aca="false">IF(B7=0,0,1-D7/B7)</f>
-        <v>0.368387853104032</v>
-      </c>
-      <c r="H7" s="17" t="n">
+        <v>0.525650737218315</v>
+      </c>
+      <c r="H7" s="21" t="n">
         <f aca="false">IF(C7=0,0,(E7-C7)/C7)</f>
-        <v>-0.404684829914757</v>
-      </c>
-      <c r="I7" s="17" t="n">
+        <v>0.0895748165123814</v>
+      </c>
+      <c r="I7" s="21" t="n">
         <f aca="false">IF(D7=0,0,(E7-D7)/D7)</f>
-        <v>-0.276471770602003</v>
+        <v>0.503065157216466</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1281,32 +1312,32 @@
         <v>50</v>
       </c>
       <c r="B8" s="14" t="n">
-        <v>540610.875</v>
+        <v>3183882.555</v>
       </c>
       <c r="C8" s="15" t="n">
-        <v>284545.536548016</v>
+        <v>2444083.52602817</v>
       </c>
       <c r="D8" s="15" t="n">
-        <v>156012.411548016</v>
+        <v>2010978.89602817</v>
       </c>
       <c r="E8" s="14" t="n">
-        <v>370000</v>
+        <v>1455000</v>
       </c>
       <c r="F8" s="16" t="n">
         <f aca="false">IF(B8=0,0,1-C8/B8)</f>
-        <v>0.473659244187391</v>
+        <v>0.232357511997433</v>
       </c>
       <c r="G8" s="16" t="n">
         <f aca="false">IF(B8=0,0,1-D8/B8)</f>
-        <v>0.711414589009117</v>
+        <v>0.368387853104032</v>
       </c>
       <c r="H8" s="17" t="n">
         <f aca="false">IF(C8=0,0,(E8-C8)/C8)</f>
-        <v>0.300319114081636</v>
+        <v>-0.404684829914757</v>
       </c>
       <c r="I8" s="17" t="n">
         <f aca="false">IF(D8=0,0,(E8-D8)/D8)</f>
-        <v>1.37160618394854</v>
+        <v>-0.276471770602003</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1314,214 +1345,258 @@
         <v>51</v>
       </c>
       <c r="B9" s="14" t="n">
-        <v>775079.55</v>
+        <v>540610.875</v>
       </c>
       <c r="C9" s="15" t="n">
-        <v>490533.729962928</v>
+        <v>284545.536548016</v>
       </c>
       <c r="D9" s="15" t="n">
-        <v>343643.979962928</v>
+        <v>156012.411548016</v>
       </c>
       <c r="E9" s="14" t="n">
-        <v>102000</v>
+        <v>370000</v>
       </c>
       <c r="F9" s="16" t="n">
         <f aca="false">IF(B9=0,0,1-C9/B9)</f>
-        <v>0.367118213913749</v>
+        <v>0.473659244187391</v>
       </c>
       <c r="G9" s="16" t="n">
         <f aca="false">IF(B9=0,0,1-D9/B9)</f>
-        <v>0.556633922333613</v>
+        <v>0.711414589009117</v>
       </c>
       <c r="H9" s="17" t="n">
         <f aca="false">IF(C9=0,0,(E9-C9)/C9)</f>
-        <v>-0.792063228745333</v>
+        <v>0.300319114081636</v>
       </c>
       <c r="I9" s="17" t="n">
         <f aca="false">IF(D9=0,0,(E9-D9)/D9)</f>
+        <v>1.37160618394854</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="18" t="s">
+        <v>52</v>
+      </c>
+      <c r="B10" s="19" t="n">
+        <f aca="false">N(B8)+N(B9)</f>
+        <v>3724493.43</v>
+      </c>
+      <c r="C10" s="19" t="n">
+        <f aca="false">N(C8)+N(C9)</f>
+        <v>2728629.06257619</v>
+      </c>
+      <c r="D10" s="19" t="n">
+        <f aca="false">N(D8)+N(D9)</f>
+        <v>2166991.30757619</v>
+      </c>
+      <c r="E10" s="19" t="n">
+        <f aca="false">N(E8)+N(E9)</f>
+        <v>1825000</v>
+      </c>
+      <c r="F10" s="20" t="n">
+        <f aca="false">IF(B10=0,0,1-C10/B10)</f>
+        <v>0.267382500772411</v>
+      </c>
+      <c r="G10" s="20" t="n">
+        <f aca="false">IF(B10=0,0,1-D10/B10)</f>
+        <v>0.418178244020641</v>
+      </c>
+      <c r="H10" s="21" t="n">
+        <f aca="false">IF(C10=0,0,(E10-C10)/C10)</f>
+        <v>-0.331165959847632</v>
+      </c>
+      <c r="I10" s="21" t="n">
+        <f aca="false">IF(D10=0,0,(E10-D10)/D10)</f>
+        <v>-0.15781849533984</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="13" t="s">
+        <v>53</v>
+      </c>
+      <c r="B11" s="14" t="n">
+        <v>775079.55</v>
+      </c>
+      <c r="C11" s="15" t="n">
+        <v>490533.729962928</v>
+      </c>
+      <c r="D11" s="15" t="n">
+        <v>343643.979962928</v>
+      </c>
+      <c r="E11" s="14" t="n">
+        <v>102000</v>
+      </c>
+      <c r="F11" s="16" t="n">
+        <f aca="false">IF(B11=0,0,1-C11/B11)</f>
+        <v>0.367118213913749</v>
+      </c>
+      <c r="G11" s="16" t="n">
+        <f aca="false">IF(B11=0,0,1-D11/B11)</f>
+        <v>0.556633922333613</v>
+      </c>
+      <c r="H11" s="17" t="n">
+        <f aca="false">IF(C11=0,0,(E11-C11)/C11)</f>
+        <v>-0.792063228745333</v>
+      </c>
+      <c r="I11" s="17" t="n">
+        <f aca="false">IF(D11=0,0,(E11-D11)/D11)</f>
         <v>-0.703181181841149</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="13" t="s">
-        <v>52</v>
-      </c>
-      <c r="B10" s="14" t="n">
+    <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="13" t="s">
+        <v>54</v>
+      </c>
+      <c r="B12" s="14" t="n">
         <v>493905.3</v>
       </c>
-      <c r="C10" s="15" t="n">
+      <c r="C12" s="15" t="n">
         <v>341463.659377819</v>
       </c>
-      <c r="D10" s="15" t="n">
+      <c r="D12" s="15" t="n">
         <v>285015.659377819</v>
       </c>
-      <c r="E10" s="14" t="n">
+      <c r="E12" s="14" t="n">
         <v>73000</v>
       </c>
-      <c r="F10" s="16" t="n">
-        <f aca="false">IF(B10=0,0,1-C10/B10)</f>
+      <c r="F12" s="16" t="n">
+        <f aca="false">IF(B12=0,0,1-C12/B12)</f>
         <v>0.308645484513288</v>
       </c>
-      <c r="G10" s="16" t="n">
-        <f aca="false">IF(B10=0,0,1-D10/B10)</f>
+      <c r="G12" s="16" t="n">
+        <f aca="false">IF(B12=0,0,1-D12/B12)</f>
         <v>0.422934600260781</v>
       </c>
-      <c r="H10" s="17" t="n">
-        <f aca="false">IF(C10=0,0,(E10-C10)/C10)</f>
+      <c r="H12" s="17" t="n">
+        <f aca="false">IF(C12=0,0,(E12-C12)/C12)</f>
         <v>-0.786214438944943</v>
       </c>
-      <c r="I10" s="17" t="n">
-        <f aca="false">IF(D10=0,0,(E10-D10)/D10)</f>
+      <c r="I12" s="17" t="n">
+        <f aca="false">IF(D12=0,0,(E12-D12)/D12)</f>
         <v>-0.743873722028618</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="18" t="s">
-        <v>53</v>
-      </c>
-      <c r="B11" s="19" t="n">
-        <f aca="false">SUM(B4:B10)</f>
+    <row r="13" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="18" t="s">
+        <v>55</v>
+      </c>
+      <c r="B13" s="19" t="n">
+        <f aca="false">N(B11)+N(B12)</f>
+        <v>1268984.85</v>
+      </c>
+      <c r="C13" s="19" t="n">
+        <f aca="false">N(C11)+N(C12)</f>
+        <v>831997.389340747</v>
+      </c>
+      <c r="D13" s="19" t="n">
+        <f aca="false">N(D11)+N(D12)</f>
+        <v>628659.639340747</v>
+      </c>
+      <c r="E13" s="19" t="n">
+        <f aca="false">N(E11)+N(E12)</f>
+        <v>175000</v>
+      </c>
+      <c r="F13" s="20" t="n">
+        <f aca="false">IF(B13=0,0,1-C13/B13)</f>
+        <v>0.344359872112936</v>
+      </c>
+      <c r="G13" s="20" t="n">
+        <f aca="false">IF(B13=0,0,1-D13/B13)</f>
+        <v>0.50459641867218</v>
+      </c>
+      <c r="H13" s="21" t="n">
+        <f aca="false">IF(C13=0,0,(E13-C13)/C13)</f>
+        <v>-0.78966280153996</v>
+      </c>
+      <c r="I13" s="21" t="n">
+        <f aca="false">IF(D13=0,0,(E13-D13)/D13)</f>
+        <v>-0.721629974236112</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="22" t="s">
+        <v>56</v>
+      </c>
+      <c r="B14" s="23" t="n">
+        <f aca="false">N(B4)+N(B5)+N(B6)+N(B8)+N(B9)+N(B11)+N(B12)</f>
         <v>7530724.005</v>
       </c>
-      <c r="C11" s="19" t="n">
-        <f aca="false">SUM(C4:C10)</f>
+      <c r="C14" s="23" t="n">
+        <f aca="false">N(C4)+N(C5)+N(C6)+N(C8)+N(C9)+N(C11)+N(C12)</f>
         <v>5220907.11606667</v>
       </c>
-      <c r="D11" s="19" t="n">
-        <f aca="false">SUM(D4:D10)</f>
+      <c r="D14" s="23" t="n">
+        <f aca="false">N(D4)+N(D5)+N(D6)+N(D8)+N(D9)+N(D11)+N(D12)</f>
         <v>3999191.58606667</v>
       </c>
-      <c r="E11" s="19" t="n">
-        <f aca="false">SUM(E4:E10)</f>
+      <c r="E14" s="23" t="n">
+        <f aca="false">N(E4)+N(E5)+N(E6)+N(E8)+N(E9)+N(E11)+N(E12)</f>
         <v>3809000</v>
       </c>
-      <c r="F11" s="20" t="n">
-        <f aca="false">IF(B11=0,0,1-C11/B11)</f>
+      <c r="F14" s="24" t="n">
+        <f aca="false">IF(B14=0,0,1-C14/B14)</f>
         <v>0.306719099969636</v>
       </c>
-      <c r="G11" s="20" t="n">
-        <f aca="false">IF(B11=0,0,1-D11/B11)</f>
+      <c r="G14" s="24" t="n">
+        <f aca="false">IF(B14=0,0,1-D14/B14)</f>
         <v>0.468949919899944</v>
       </c>
-      <c r="H11" s="21" t="n">
-        <f aca="false">IF(C11=0,0,(E11-C11)/C11)</f>
+      <c r="H14" s="25" t="n">
+        <f aca="false">IF(C14=0,0,(E14-C14)/C14)</f>
         <v>-0.2704332953409</v>
       </c>
-      <c r="I11" s="21" t="n">
-        <f aca="false">IF(D11=0,0,(E11-D11)/D11)</f>
+      <c r="I14" s="25" t="n">
+        <f aca="false">IF(D14=0,0,(E14-D14)/D14)</f>
         <v>-0.047557508054703</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="22"/>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="12" t="s">
-        <v>54</v>
-      </c>
-      <c r="B13" s="12"/>
-      <c r="C13" s="12"/>
-      <c r="D13" s="12"/>
-      <c r="E13" s="12"/>
-      <c r="F13" s="12"/>
-      <c r="G13" s="12"/>
-      <c r="H13" s="12"/>
-      <c r="I13" s="12"/>
-    </row>
-    <row r="14" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="3" t="s">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="B16" s="12"/>
+      <c r="C16" s="12"/>
+      <c r="D16" s="12"/>
+      <c r="E16" s="12"/>
+      <c r="F16" s="12"/>
+      <c r="G16" s="12"/>
+      <c r="H16" s="12"/>
+      <c r="I16" s="12"/>
+    </row>
+    <row r="17" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="B14" s="3" t="s">
+      <c r="B17" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="C14" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="D14" s="3" t="s">
+      <c r="C17" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="D17" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="E14" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="F14" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="G14" s="3" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="13" t="s">
-        <v>24</v>
-      </c>
-      <c r="B15" s="23"/>
-      <c r="C15" s="23"/>
-      <c r="D15" s="15" t="n">
-        <f aca="false">N(B15)-N(C15)</f>
-        <v>0</v>
-      </c>
-      <c r="E15" s="23"/>
-      <c r="F15" s="16" t="n">
-        <f aca="false">IF(N(B15)=0,0,1-D15/B15)</f>
-        <v>0</v>
-      </c>
-      <c r="G15" s="17" t="n">
-        <f aca="false">IF(D15=0,0,(N(E15)-D15)/D15)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="13" t="s">
-        <v>13</v>
-      </c>
-      <c r="B16" s="23"/>
-      <c r="C16" s="23"/>
-      <c r="D16" s="15" t="n">
-        <f aca="false">N(B16)-N(C16)</f>
-        <v>0</v>
-      </c>
-      <c r="E16" s="23"/>
-      <c r="F16" s="16" t="n">
-        <f aca="false">IF(N(B16)=0,0,1-D16/B16)</f>
-        <v>0</v>
-      </c>
-      <c r="G16" s="17" t="n">
-        <f aca="false">IF(D16=0,0,(N(E16)-D16)/D16)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="13" t="s">
-        <v>48</v>
-      </c>
-      <c r="B17" s="23"/>
-      <c r="C17" s="23"/>
-      <c r="D17" s="15" t="n">
-        <f aca="false">N(B17)-N(C17)</f>
-        <v>0</v>
-      </c>
-      <c r="E17" s="23"/>
-      <c r="F17" s="16" t="n">
-        <f aca="false">IF(N(B17)=0,0,1-D17/B17)</f>
-        <v>0</v>
-      </c>
-      <c r="G17" s="17" t="n">
-        <f aca="false">IF(D17=0,0,(N(E17)-D17)/D17)</f>
-        <v>0</v>
+      <c r="E17" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="F17" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="G17" s="3" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="13" t="s">
-        <v>49</v>
-      </c>
-      <c r="B18" s="23"/>
-      <c r="C18" s="23"/>
+        <v>24</v>
+      </c>
+      <c r="B18" s="26"/>
+      <c r="C18" s="26"/>
       <c r="D18" s="15" t="n">
         <f aca="false">N(B18)-N(C18)</f>
         <v>0</v>
       </c>
-      <c r="E18" s="23"/>
+      <c r="E18" s="26"/>
       <c r="F18" s="16" t="n">
         <f aca="false">IF(N(B18)=0,0,1-D18/B18)</f>
         <v>0</v>
@@ -1533,15 +1608,15 @@
     </row>
     <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="13" t="s">
-        <v>50</v>
-      </c>
-      <c r="B19" s="23"/>
-      <c r="C19" s="23"/>
+        <v>13</v>
+      </c>
+      <c r="B19" s="26"/>
+      <c r="C19" s="26"/>
       <c r="D19" s="15" t="n">
         <f aca="false">N(B19)-N(C19)</f>
         <v>0</v>
       </c>
-      <c r="E19" s="23"/>
+      <c r="E19" s="26"/>
       <c r="F19" s="16" t="n">
         <f aca="false">IF(N(B19)=0,0,1-D19/B19)</f>
         <v>0</v>
@@ -1553,15 +1628,15 @@
     </row>
     <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="13" t="s">
-        <v>51</v>
-      </c>
-      <c r="B20" s="23"/>
-      <c r="C20" s="23"/>
+        <v>48</v>
+      </c>
+      <c r="B20" s="26"/>
+      <c r="C20" s="26"/>
       <c r="D20" s="15" t="n">
         <f aca="false">N(B20)-N(C20)</f>
         <v>0</v>
       </c>
-      <c r="E20" s="23"/>
+      <c r="E20" s="26"/>
       <c r="F20" s="16" t="n">
         <f aca="false">IF(N(B20)=0,0,1-D20/B20)</f>
         <v>0</v>
@@ -1571,539 +1646,797 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="13" t="s">
+    <row r="21" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="18" t="s">
+        <v>49</v>
+      </c>
+      <c r="B21" s="19" t="n">
+        <f aca="false">N(B18)+N(B19)+N(B20)</f>
+        <v>0</v>
+      </c>
+      <c r="C21" s="19" t="n">
+        <f aca="false">N(C18)+N(C19)+N(C20)</f>
+        <v>0</v>
+      </c>
+      <c r="D21" s="19" t="n">
+        <f aca="false">N(D18)+N(D19)+N(D20)</f>
+        <v>0</v>
+      </c>
+      <c r="E21" s="19" t="n">
+        <f aca="false">N(E18)+N(E19)+N(E20)</f>
+        <v>0</v>
+      </c>
+      <c r="F21" s="20" t="n">
+        <f aca="false">IF(N(B21)=0,0,1-D21/B21)</f>
+        <v>0</v>
+      </c>
+      <c r="G21" s="21" t="n">
+        <f aca="false">IF(D21=0,0,(N(E21)-D21)/D21)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="B22" s="26"/>
+      <c r="C22" s="26"/>
+      <c r="D22" s="15" t="n">
+        <f aca="false">N(B22)-N(C22)</f>
+        <v>0</v>
+      </c>
+      <c r="E22" s="26"/>
+      <c r="F22" s="16" t="n">
+        <f aca="false">IF(N(B22)=0,0,1-D22/B22)</f>
+        <v>0</v>
+      </c>
+      <c r="G22" s="17" t="n">
+        <f aca="false">IF(D22=0,0,(N(E22)-D22)/D22)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="13" t="s">
+        <v>51</v>
+      </c>
+      <c r="B23" s="26"/>
+      <c r="C23" s="26"/>
+      <c r="D23" s="15" t="n">
+        <f aca="false">N(B23)-N(C23)</f>
+        <v>0</v>
+      </c>
+      <c r="E23" s="26"/>
+      <c r="F23" s="16" t="n">
+        <f aca="false">IF(N(B23)=0,0,1-D23/B23)</f>
+        <v>0</v>
+      </c>
+      <c r="G23" s="17" t="n">
+        <f aca="false">IF(D23=0,0,(N(E23)-D23)/D23)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="18" t="s">
         <v>52</v>
       </c>
-      <c r="B21" s="23"/>
-      <c r="C21" s="23"/>
-      <c r="D21" s="15" t="n">
-        <f aca="false">N(B21)-N(C21)</f>
-        <v>0</v>
-      </c>
-      <c r="E21" s="23"/>
-      <c r="F21" s="16" t="n">
-        <f aca="false">IF(N(B21)=0,0,1-D21/B21)</f>
-        <v>0</v>
-      </c>
-      <c r="G21" s="17" t="n">
-        <f aca="false">IF(D21=0,0,(N(E21)-D21)/D21)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="18" t="s">
+      <c r="B24" s="19" t="n">
+        <f aca="false">N(B22)+N(B23)</f>
+        <v>0</v>
+      </c>
+      <c r="C24" s="19" t="n">
+        <f aca="false">N(C22)+N(C23)</f>
+        <v>0</v>
+      </c>
+      <c r="D24" s="19" t="n">
+        <f aca="false">N(D22)+N(D23)</f>
+        <v>0</v>
+      </c>
+      <c r="E24" s="19" t="n">
+        <f aca="false">N(E22)+N(E23)</f>
+        <v>0</v>
+      </c>
+      <c r="F24" s="20" t="n">
+        <f aca="false">IF(N(B24)=0,0,1-D24/B24)</f>
+        <v>0</v>
+      </c>
+      <c r="G24" s="21" t="n">
+        <f aca="false">IF(D24=0,0,(N(E24)-D24)/D24)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="13" t="s">
         <v>53</v>
       </c>
-      <c r="B22" s="19" t="n">
-        <f aca="false">SUM(B15:B21)</f>
-        <v>0</v>
-      </c>
-      <c r="C22" s="19" t="n">
-        <f aca="false">SUM(C15:C21)</f>
-        <v>0</v>
-      </c>
-      <c r="D22" s="19" t="n">
-        <f aca="false">SUM(D15:D21)</f>
-        <v>0</v>
-      </c>
-      <c r="E22" s="19" t="n">
-        <f aca="false">SUM(E15:E21)</f>
-        <v>0</v>
-      </c>
-      <c r="F22" s="20" t="n">
-        <f aca="false">IF(B22=0,0,1-D22/B22)</f>
-        <v>0</v>
-      </c>
-      <c r="G22" s="21" t="n">
-        <f aca="false">IF(D22=0,0,(E22-D22)/D22)</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="2" t="str">
-        <f aca="false">IF(ROUND(C22-Reductions!D17,0)=0,"Check: Pharma discounts match the total in the Reductions tab.","Check: Pharma discounts by stage ("&amp;TEXT(C22,"#,##0")&amp;") do not match the total in the Reductions tab ("&amp;TEXT(Reductions!D17,"#,##0")&amp;").")</f>
+      <c r="B25" s="26"/>
+      <c r="C25" s="26"/>
+      <c r="D25" s="15" t="n">
+        <f aca="false">N(B25)-N(C25)</f>
+        <v>0</v>
+      </c>
+      <c r="E25" s="26"/>
+      <c r="F25" s="16" t="n">
+        <f aca="false">IF(N(B25)=0,0,1-D25/B25)</f>
+        <v>0</v>
+      </c>
+      <c r="G25" s="17" t="n">
+        <f aca="false">IF(D25=0,0,(N(E25)-D25)/D25)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="13" t="s">
+        <v>54</v>
+      </c>
+      <c r="B26" s="26"/>
+      <c r="C26" s="26"/>
+      <c r="D26" s="15" t="n">
+        <f aca="false">N(B26)-N(C26)</f>
+        <v>0</v>
+      </c>
+      <c r="E26" s="26"/>
+      <c r="F26" s="16" t="n">
+        <f aca="false">IF(N(B26)=0,0,1-D26/B26)</f>
+        <v>0</v>
+      </c>
+      <c r="G26" s="17" t="n">
+        <f aca="false">IF(D26=0,0,(N(E26)-D26)/D26)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="18" t="s">
+        <v>55</v>
+      </c>
+      <c r="B27" s="19" t="n">
+        <f aca="false">N(B25)+N(B26)</f>
+        <v>0</v>
+      </c>
+      <c r="C27" s="19" t="n">
+        <f aca="false">N(C25)+N(C26)</f>
+        <v>0</v>
+      </c>
+      <c r="D27" s="19" t="n">
+        <f aca="false">N(D25)+N(D26)</f>
+        <v>0</v>
+      </c>
+      <c r="E27" s="19" t="n">
+        <f aca="false">N(E25)+N(E26)</f>
+        <v>0</v>
+      </c>
+      <c r="F27" s="20" t="n">
+        <f aca="false">IF(N(B27)=0,0,1-D27/B27)</f>
+        <v>0</v>
+      </c>
+      <c r="G27" s="21" t="n">
+        <f aca="false">IF(D27=0,0,(N(E27)-D27)/D27)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="22" t="s">
+        <v>56</v>
+      </c>
+      <c r="B28" s="23" t="n">
+        <f aca="false">N(B18)+N(B19)+N(B20)+N(B22)+N(B23)+N(B25)+N(B26)</f>
+        <v>0</v>
+      </c>
+      <c r="C28" s="23" t="n">
+        <f aca="false">N(C18)+N(C19)+N(C20)+N(C22)+N(C23)+N(C25)+N(C26)</f>
+        <v>0</v>
+      </c>
+      <c r="D28" s="23" t="n">
+        <f aca="false">N(D18)+N(D19)+N(D20)+N(D22)+N(D23)+N(D25)+N(D26)</f>
+        <v>0</v>
+      </c>
+      <c r="E28" s="23" t="n">
+        <f aca="false">N(E18)+N(E19)+N(E20)+N(E22)+N(E23)+N(E25)+N(E26)</f>
+        <v>0</v>
+      </c>
+      <c r="F28" s="24" t="n">
+        <f aca="false">IF(N(B28)=0,0,1-D28/B28)</f>
+        <v>0</v>
+      </c>
+      <c r="G28" s="25" t="n">
+        <f aca="false">IF(D28=0,0,(N(E28)-D28)/D28)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="2" t="str">
+        <f aca="false">IF(ROUND(C28-Reductions!D17,0)=0,"Check: Pharma discounts match the total in the Reductions tab.","Check: Pharma discounts by stage ("&amp;TEXT(C28,"#,##0")&amp;") do not match the total in the Reductions tab ("&amp;TEXT(Reductions!D17,"#,##0")&amp;").")</f>
         <v>Check: Pharma discounts match the total in the Reductions tab.</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="2" t="s">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="12" t="s">
-        <v>60</v>
-      </c>
-      <c r="B26" s="12"/>
-      <c r="C26" s="12"/>
-      <c r="D26" s="12"/>
-      <c r="E26" s="12"/>
-      <c r="F26" s="12"/>
-      <c r="G26" s="12"/>
-      <c r="H26" s="12"/>
-      <c r="I26" s="12"/>
-    </row>
-    <row r="27" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="3" t="s">
+    <row r="30" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="2" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="12" t="s">
+        <v>63</v>
+      </c>
+      <c r="B32" s="12"/>
+      <c r="C32" s="12"/>
+      <c r="D32" s="12"/>
+      <c r="E32" s="12"/>
+      <c r="F32" s="12"/>
+      <c r="G32" s="12"/>
+      <c r="H32" s="12"/>
+      <c r="I32" s="12"/>
+    </row>
+    <row r="33" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="3" t="s">
         <v>39</v>
       </c>
-      <c r="B27" s="3" t="s">
+      <c r="B33" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="C27" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="D27" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="E27" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="F27" s="3" t="s">
+      <c r="C33" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="D33" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="E33" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="F33" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="G27" s="3" t="s">
+      <c r="G33" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="H27" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="I27" s="3" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="13" t="s">
-        <v>24</v>
-      </c>
-      <c r="B28" s="14" t="n">
-        <f aca="false">B4+N(B15)</f>
-        <v>335082.825</v>
-      </c>
-      <c r="C28" s="15" t="n">
-        <f aca="false">C4+D15</f>
-        <v>229164.869624349</v>
-      </c>
-      <c r="D28" s="15" t="n">
-        <f aca="false">D4+D15</f>
-        <v>121097.819624349</v>
-      </c>
-      <c r="E28" s="14" t="n">
-        <f aca="false">E4+N(E15)</f>
-        <v>106000</v>
-      </c>
-      <c r="F28" s="16" t="n">
-        <f aca="false">IF(B28=0,0,1-C28/B28)</f>
-        <v>0.316094850208008</v>
-      </c>
-      <c r="G28" s="16" t="n">
-        <f aca="false">IF(B28=0,0,1-D28/B28)</f>
-        <v>0.638603322553613</v>
-      </c>
-      <c r="H28" s="17" t="n">
-        <f aca="false">IF(C28=0,0,(E28-C28)/C28)</f>
-        <v>-0.537450918311533</v>
-      </c>
-      <c r="I28" s="17" t="n">
-        <f aca="false">IF(D28=0,0,(E28-D28)/D28)</f>
-        <v>-0.12467457854471</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="13" t="s">
-        <v>13</v>
-      </c>
-      <c r="B29" s="14" t="n">
-        <f aca="false">B5+N(B16)</f>
-        <v>732839.1</v>
-      </c>
-      <c r="C29" s="15" t="n">
-        <f aca="false">C5+D16</f>
-        <v>294268.667883964</v>
-      </c>
-      <c r="D29" s="15" t="n">
-        <f aca="false">D5+D16</f>
-        <v>135402.092883964</v>
-      </c>
-      <c r="E29" s="14" t="n">
-        <f aca="false">E5+N(E16)</f>
-        <v>453000</v>
-      </c>
-      <c r="F29" s="16" t="n">
-        <f aca="false">IF(B29=0,0,1-C29/B29)</f>
-        <v>0.598453919988762</v>
-      </c>
-      <c r="G29" s="16" t="n">
-        <f aca="false">IF(B29=0,0,1-D29/B29)</f>
-        <v>0.815236260068596</v>
-      </c>
-      <c r="H29" s="17" t="n">
-        <f aca="false">IF(C29=0,0,(E29-C29)/C29)</f>
-        <v>0.539409558134225</v>
-      </c>
-      <c r="I29" s="17" t="n">
-        <f aca="false">IF(D29=0,0,(E29-D29)/D29)</f>
-        <v>2.34559082767065</v>
-      </c>
-    </row>
-    <row r="30" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="13" t="s">
-        <v>48</v>
-      </c>
-      <c r="B30" s="14" t="n">
-        <f aca="false">B6+N(B17)</f>
-        <v>1469323.8</v>
-      </c>
-      <c r="C30" s="15" t="n">
-        <f aca="false">C6+D17</f>
-        <v>1136847.12664142</v>
-      </c>
-      <c r="D30" s="15" t="n">
-        <f aca="false">D6+D17</f>
-        <v>947040.72664142</v>
-      </c>
-      <c r="E30" s="14" t="n">
-        <f aca="false">E6+N(E17)</f>
-        <v>1250000</v>
-      </c>
-      <c r="F30" s="16" t="n">
-        <f aca="false">IF(B30=0,0,1-C30/B30)</f>
-        <v>0.226278695927052</v>
-      </c>
-      <c r="G30" s="16" t="n">
-        <f aca="false">IF(B30=0,0,1-D30/B30)</f>
-        <v>0.355458118461417</v>
-      </c>
-      <c r="H30" s="17" t="n">
-        <f aca="false">IF(C30=0,0,(E30-C30)/C30)</f>
-        <v>0.0995321804549631</v>
-      </c>
-      <c r="I30" s="17" t="n">
-        <f aca="false">IF(D30=0,0,(E30-D30)/D30)</f>
-        <v>0.319900997745887</v>
-      </c>
-    </row>
-    <row r="31" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="13" t="s">
-        <v>49</v>
-      </c>
-      <c r="B31" s="14" t="n">
-        <f aca="false">B7+N(B18)</f>
-        <v>3183882.555</v>
-      </c>
-      <c r="C31" s="15" t="n">
-        <f aca="false">C7+D18</f>
-        <v>2444083.52602817</v>
-      </c>
-      <c r="D31" s="15" t="n">
-        <f aca="false">D7+D18</f>
-        <v>2010978.89602817</v>
-      </c>
-      <c r="E31" s="14" t="n">
-        <f aca="false">E7+N(E18)</f>
-        <v>1455000</v>
-      </c>
-      <c r="F31" s="16" t="n">
-        <f aca="false">IF(B31=0,0,1-C31/B31)</f>
-        <v>0.232357511997433</v>
-      </c>
-      <c r="G31" s="16" t="n">
-        <f aca="false">IF(B31=0,0,1-D31/B31)</f>
-        <v>0.368387853104032</v>
-      </c>
-      <c r="H31" s="17" t="n">
-        <f aca="false">IF(C31=0,0,(E31-C31)/C31)</f>
-        <v>-0.404684829914757</v>
-      </c>
-      <c r="I31" s="17" t="n">
-        <f aca="false">IF(D31=0,0,(E31-D31)/D31)</f>
-        <v>-0.276471770602003</v>
-      </c>
-    </row>
-    <row r="32" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="13" t="s">
-        <v>50</v>
-      </c>
-      <c r="B32" s="14" t="n">
-        <f aca="false">B8+N(B19)</f>
-        <v>540610.875</v>
-      </c>
-      <c r="C32" s="15" t="n">
-        <f aca="false">C8+D19</f>
-        <v>284545.536548016</v>
-      </c>
-      <c r="D32" s="15" t="n">
-        <f aca="false">D8+D19</f>
-        <v>156012.411548016</v>
-      </c>
-      <c r="E32" s="14" t="n">
-        <f aca="false">E8+N(E19)</f>
-        <v>370000</v>
-      </c>
-      <c r="F32" s="16" t="n">
-        <f aca="false">IF(B32=0,0,1-C32/B32)</f>
-        <v>0.473659244187391</v>
-      </c>
-      <c r="G32" s="16" t="n">
-        <f aca="false">IF(B32=0,0,1-D32/B32)</f>
-        <v>0.711414589009117</v>
-      </c>
-      <c r="H32" s="17" t="n">
-        <f aca="false">IF(C32=0,0,(E32-C32)/C32)</f>
-        <v>0.300319114081636</v>
-      </c>
-      <c r="I32" s="17" t="n">
-        <f aca="false">IF(D32=0,0,(E32-D32)/D32)</f>
-        <v>1.37160618394854</v>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="13" t="s">
-        <v>51</v>
-      </c>
-      <c r="B33" s="14" t="n">
-        <f aca="false">B9+N(B20)</f>
-        <v>775079.55</v>
-      </c>
-      <c r="C33" s="15" t="n">
-        <f aca="false">C9+D20</f>
-        <v>490533.729962928</v>
-      </c>
-      <c r="D33" s="15" t="n">
-        <f aca="false">D9+D20</f>
-        <v>343643.979962928</v>
-      </c>
-      <c r="E33" s="14" t="n">
-        <f aca="false">E9+N(E20)</f>
-        <v>102000</v>
-      </c>
-      <c r="F33" s="16" t="n">
-        <f aca="false">IF(B33=0,0,1-C33/B33)</f>
-        <v>0.367118213913749</v>
-      </c>
-      <c r="G33" s="16" t="n">
-        <f aca="false">IF(B33=0,0,1-D33/B33)</f>
-        <v>0.556633922333613</v>
-      </c>
-      <c r="H33" s="17" t="n">
-        <f aca="false">IF(C33=0,0,(E33-C33)/C33)</f>
-        <v>-0.792063228745333</v>
-      </c>
-      <c r="I33" s="17" t="n">
-        <f aca="false">IF(D33=0,0,(E33-D33)/D33)</f>
-        <v>-0.703181181841149</v>
+      <c r="H33" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="I33" s="3" t="s">
+        <v>68</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="13" t="s">
-        <v>52</v>
+        <v>24</v>
       </c>
       <c r="B34" s="14" t="n">
-        <f aca="false">B10+N(B21)</f>
-        <v>493905.3</v>
+        <f aca="false">B4+N(B18)</f>
+        <v>335082.825</v>
       </c>
       <c r="C34" s="15" t="n">
-        <f aca="false">C10+D21</f>
-        <v>341463.659377819</v>
+        <f aca="false">C4+D18</f>
+        <v>229164.869624349</v>
       </c>
       <c r="D34" s="15" t="n">
-        <f aca="false">D10+D21</f>
-        <v>285015.659377819</v>
+        <f aca="false">D4+D18</f>
+        <v>121097.819624349</v>
       </c>
       <c r="E34" s="14" t="n">
-        <f aca="false">E10+N(E21)</f>
-        <v>73000</v>
+        <f aca="false">E4+N(E18)</f>
+        <v>106000</v>
       </c>
       <c r="F34" s="16" t="n">
         <f aca="false">IF(B34=0,0,1-C34/B34)</f>
-        <v>0.308645484513288</v>
+        <v>0.316094850208008</v>
       </c>
       <c r="G34" s="16" t="n">
         <f aca="false">IF(B34=0,0,1-D34/B34)</f>
-        <v>0.422934600260781</v>
+        <v>0.638603322553613</v>
       </c>
       <c r="H34" s="17" t="n">
         <f aca="false">IF(C34=0,0,(E34-C34)/C34)</f>
-        <v>-0.786214438944943</v>
+        <v>-0.537450918311533</v>
       </c>
       <c r="I34" s="17" t="n">
         <f aca="false">IF(D34=0,0,(E34-D34)/D34)</f>
+        <v>-0.12467457854471</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A35" s="13" t="s">
+        <v>13</v>
+      </c>
+      <c r="B35" s="14" t="n">
+        <f aca="false">B5+N(B19)</f>
+        <v>732839.1</v>
+      </c>
+      <c r="C35" s="15" t="n">
+        <f aca="false">C5+D19</f>
+        <v>294268.667883964</v>
+      </c>
+      <c r="D35" s="15" t="n">
+        <f aca="false">D5+D19</f>
+        <v>135402.092883964</v>
+      </c>
+      <c r="E35" s="14" t="n">
+        <f aca="false">E5+N(E19)</f>
+        <v>453000</v>
+      </c>
+      <c r="F35" s="16" t="n">
+        <f aca="false">IF(B35=0,0,1-C35/B35)</f>
+        <v>0.598453919988762</v>
+      </c>
+      <c r="G35" s="16" t="n">
+        <f aca="false">IF(B35=0,0,1-D35/B35)</f>
+        <v>0.815236260068596</v>
+      </c>
+      <c r="H35" s="17" t="n">
+        <f aca="false">IF(C35=0,0,(E35-C35)/C35)</f>
+        <v>0.539409558134225</v>
+      </c>
+      <c r="I35" s="17" t="n">
+        <f aca="false">IF(D35=0,0,(E35-D35)/D35)</f>
+        <v>2.34559082767065</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="13" t="s">
+        <v>48</v>
+      </c>
+      <c r="B36" s="14" t="n">
+        <f aca="false">B6+N(B20)</f>
+        <v>1469323.8</v>
+      </c>
+      <c r="C36" s="15" t="n">
+        <f aca="false">C6+D20</f>
+        <v>1136847.12664142</v>
+      </c>
+      <c r="D36" s="15" t="n">
+        <f aca="false">D6+D20</f>
+        <v>947040.72664142</v>
+      </c>
+      <c r="E36" s="14" t="n">
+        <f aca="false">E6+N(E20)</f>
+        <v>1250000</v>
+      </c>
+      <c r="F36" s="16" t="n">
+        <f aca="false">IF(B36=0,0,1-C36/B36)</f>
+        <v>0.226278695927052</v>
+      </c>
+      <c r="G36" s="16" t="n">
+        <f aca="false">IF(B36=0,0,1-D36/B36)</f>
+        <v>0.355458118461417</v>
+      </c>
+      <c r="H36" s="17" t="n">
+        <f aca="false">IF(C36=0,0,(E36-C36)/C36)</f>
+        <v>0.0995321804549631</v>
+      </c>
+      <c r="I36" s="17" t="n">
+        <f aca="false">IF(D36=0,0,(E36-D36)/D36)</f>
+        <v>0.319900997745887</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A37" s="18" t="s">
+        <v>49</v>
+      </c>
+      <c r="B37" s="19" t="n">
+        <f aca="false">N(B34)+N(B35)+N(B36)</f>
+        <v>2537245.725</v>
+      </c>
+      <c r="C37" s="19" t="n">
+        <f aca="false">N(C34)+N(C35)+N(C36)</f>
+        <v>1660280.66414973</v>
+      </c>
+      <c r="D37" s="19" t="n">
+        <f aca="false">N(D34)+N(D35)+N(D36)</f>
+        <v>1203540.63914973</v>
+      </c>
+      <c r="E37" s="19" t="n">
+        <f aca="false">N(E34)+N(E35)+N(E36)</f>
+        <v>1809000</v>
+      </c>
+      <c r="F37" s="20" t="n">
+        <f aca="false">IF(B37=0,0,1-C37/B37)</f>
+        <v>0.345636629597737</v>
+      </c>
+      <c r="G37" s="20" t="n">
+        <f aca="false">IF(B37=0,0,1-D37/B37)</f>
+        <v>0.525650737218315</v>
+      </c>
+      <c r="H37" s="21" t="n">
+        <f aca="false">IF(C37=0,0,(E37-C37)/C37)</f>
+        <v>0.0895748165123814</v>
+      </c>
+      <c r="I37" s="21" t="n">
+        <f aca="false">IF(D37=0,0,(E37-D37)/D37)</f>
+        <v>0.503065157216466</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A38" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="B38" s="14" t="n">
+        <f aca="false">B8+N(B22)</f>
+        <v>3183882.555</v>
+      </c>
+      <c r="C38" s="15" t="n">
+        <f aca="false">C8+D22</f>
+        <v>2444083.52602817</v>
+      </c>
+      <c r="D38" s="15" t="n">
+        <f aca="false">D8+D22</f>
+        <v>2010978.89602817</v>
+      </c>
+      <c r="E38" s="14" t="n">
+        <f aca="false">E8+N(E22)</f>
+        <v>1455000</v>
+      </c>
+      <c r="F38" s="16" t="n">
+        <f aca="false">IF(B38=0,0,1-C38/B38)</f>
+        <v>0.232357511997433</v>
+      </c>
+      <c r="G38" s="16" t="n">
+        <f aca="false">IF(B38=0,0,1-D38/B38)</f>
+        <v>0.368387853104032</v>
+      </c>
+      <c r="H38" s="17" t="n">
+        <f aca="false">IF(C38=0,0,(E38-C38)/C38)</f>
+        <v>-0.404684829914757</v>
+      </c>
+      <c r="I38" s="17" t="n">
+        <f aca="false">IF(D38=0,0,(E38-D38)/D38)</f>
+        <v>-0.276471770602003</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A39" s="13" t="s">
+        <v>51</v>
+      </c>
+      <c r="B39" s="14" t="n">
+        <f aca="false">B9+N(B23)</f>
+        <v>540610.875</v>
+      </c>
+      <c r="C39" s="15" t="n">
+        <f aca="false">C9+D23</f>
+        <v>284545.536548016</v>
+      </c>
+      <c r="D39" s="15" t="n">
+        <f aca="false">D9+D23</f>
+        <v>156012.411548016</v>
+      </c>
+      <c r="E39" s="14" t="n">
+        <f aca="false">E9+N(E23)</f>
+        <v>370000</v>
+      </c>
+      <c r="F39" s="16" t="n">
+        <f aca="false">IF(B39=0,0,1-C39/B39)</f>
+        <v>0.473659244187391</v>
+      </c>
+      <c r="G39" s="16" t="n">
+        <f aca="false">IF(B39=0,0,1-D39/B39)</f>
+        <v>0.711414589009117</v>
+      </c>
+      <c r="H39" s="17" t="n">
+        <f aca="false">IF(C39=0,0,(E39-C39)/C39)</f>
+        <v>0.300319114081636</v>
+      </c>
+      <c r="I39" s="17" t="n">
+        <f aca="false">IF(D39=0,0,(E39-D39)/D39)</f>
+        <v>1.37160618394854</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A40" s="18" t="s">
+        <v>52</v>
+      </c>
+      <c r="B40" s="19" t="n">
+        <f aca="false">N(B38)+N(B39)</f>
+        <v>3724493.43</v>
+      </c>
+      <c r="C40" s="19" t="n">
+        <f aca="false">N(C38)+N(C39)</f>
+        <v>2728629.06257619</v>
+      </c>
+      <c r="D40" s="19" t="n">
+        <f aca="false">N(D38)+N(D39)</f>
+        <v>2166991.30757619</v>
+      </c>
+      <c r="E40" s="19" t="n">
+        <f aca="false">N(E38)+N(E39)</f>
+        <v>1825000</v>
+      </c>
+      <c r="F40" s="20" t="n">
+        <f aca="false">IF(B40=0,0,1-C40/B40)</f>
+        <v>0.267382500772411</v>
+      </c>
+      <c r="G40" s="20" t="n">
+        <f aca="false">IF(B40=0,0,1-D40/B40)</f>
+        <v>0.418178244020641</v>
+      </c>
+      <c r="H40" s="21" t="n">
+        <f aca="false">IF(C40=0,0,(E40-C40)/C40)</f>
+        <v>-0.331165959847632</v>
+      </c>
+      <c r="I40" s="21" t="n">
+        <f aca="false">IF(D40=0,0,(E40-D40)/D40)</f>
+        <v>-0.15781849533984</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A41" s="13" t="s">
+        <v>53</v>
+      </c>
+      <c r="B41" s="14" t="n">
+        <f aca="false">B11+N(B25)</f>
+        <v>775079.55</v>
+      </c>
+      <c r="C41" s="15" t="n">
+        <f aca="false">C11+D25</f>
+        <v>490533.729962928</v>
+      </c>
+      <c r="D41" s="15" t="n">
+        <f aca="false">D11+D25</f>
+        <v>343643.979962928</v>
+      </c>
+      <c r="E41" s="14" t="n">
+        <f aca="false">E11+N(E25)</f>
+        <v>102000</v>
+      </c>
+      <c r="F41" s="16" t="n">
+        <f aca="false">IF(B41=0,0,1-C41/B41)</f>
+        <v>0.367118213913749</v>
+      </c>
+      <c r="G41" s="16" t="n">
+        <f aca="false">IF(B41=0,0,1-D41/B41)</f>
+        <v>0.556633922333613</v>
+      </c>
+      <c r="H41" s="17" t="n">
+        <f aca="false">IF(C41=0,0,(E41-C41)/C41)</f>
+        <v>-0.792063228745333</v>
+      </c>
+      <c r="I41" s="17" t="n">
+        <f aca="false">IF(D41=0,0,(E41-D41)/D41)</f>
+        <v>-0.703181181841149</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A42" s="13" t="s">
+        <v>54</v>
+      </c>
+      <c r="B42" s="14" t="n">
+        <f aca="false">B12+N(B26)</f>
+        <v>493905.3</v>
+      </c>
+      <c r="C42" s="15" t="n">
+        <f aca="false">C12+D26</f>
+        <v>341463.659377819</v>
+      </c>
+      <c r="D42" s="15" t="n">
+        <f aca="false">D12+D26</f>
+        <v>285015.659377819</v>
+      </c>
+      <c r="E42" s="14" t="n">
+        <f aca="false">E12+N(E26)</f>
+        <v>73000</v>
+      </c>
+      <c r="F42" s="16" t="n">
+        <f aca="false">IF(B42=0,0,1-C42/B42)</f>
+        <v>0.308645484513288</v>
+      </c>
+      <c r="G42" s="16" t="n">
+        <f aca="false">IF(B42=0,0,1-D42/B42)</f>
+        <v>0.422934600260781</v>
+      </c>
+      <c r="H42" s="17" t="n">
+        <f aca="false">IF(C42=0,0,(E42-C42)/C42)</f>
+        <v>-0.786214438944943</v>
+      </c>
+      <c r="I42" s="17" t="n">
+        <f aca="false">IF(D42=0,0,(E42-D42)/D42)</f>
         <v>-0.743873722028618</v>
       </c>
     </row>
-    <row r="35" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A35" s="18" t="s">
-        <v>53</v>
-      </c>
-      <c r="B35" s="19" t="n">
-        <f aca="false">SUM(B28:B34)</f>
+    <row r="43" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A43" s="18" t="s">
+        <v>55</v>
+      </c>
+      <c r="B43" s="19" t="n">
+        <f aca="false">N(B41)+N(B42)</f>
+        <v>1268984.85</v>
+      </c>
+      <c r="C43" s="19" t="n">
+        <f aca="false">N(C41)+N(C42)</f>
+        <v>831997.389340747</v>
+      </c>
+      <c r="D43" s="19" t="n">
+        <f aca="false">N(D41)+N(D42)</f>
+        <v>628659.639340747</v>
+      </c>
+      <c r="E43" s="19" t="n">
+        <f aca="false">N(E41)+N(E42)</f>
+        <v>175000</v>
+      </c>
+      <c r="F43" s="20" t="n">
+        <f aca="false">IF(B43=0,0,1-C43/B43)</f>
+        <v>0.344359872112936</v>
+      </c>
+      <c r="G43" s="20" t="n">
+        <f aca="false">IF(B43=0,0,1-D43/B43)</f>
+        <v>0.50459641867218</v>
+      </c>
+      <c r="H43" s="21" t="n">
+        <f aca="false">IF(C43=0,0,(E43-C43)/C43)</f>
+        <v>-0.78966280153996</v>
+      </c>
+      <c r="I43" s="21" t="n">
+        <f aca="false">IF(D43=0,0,(E43-D43)/D43)</f>
+        <v>-0.721629974236112</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A44" s="22" t="s">
+        <v>56</v>
+      </c>
+      <c r="B44" s="23" t="n">
+        <f aca="false">N(B34)+N(B35)+N(B36)+N(B38)+N(B39)+N(B41)+N(B42)</f>
         <v>7530724.005</v>
       </c>
-      <c r="C35" s="19" t="n">
-        <f aca="false">SUM(C28:C34)</f>
+      <c r="C44" s="23" t="n">
+        <f aca="false">N(C34)+N(C35)+N(C36)+N(C38)+N(C39)+N(C41)+N(C42)</f>
         <v>5220907.11606667</v>
       </c>
-      <c r="D35" s="19" t="n">
-        <f aca="false">SUM(D28:D34)</f>
+      <c r="D44" s="23" t="n">
+        <f aca="false">N(D34)+N(D35)+N(D36)+N(D38)+N(D39)+N(D41)+N(D42)</f>
         <v>3999191.58606667</v>
       </c>
-      <c r="E35" s="19" t="n">
-        <f aca="false">SUM(E28:E34)</f>
+      <c r="E44" s="23" t="n">
+        <f aca="false">N(E34)+N(E35)+N(E36)+N(E38)+N(E39)+N(E41)+N(E42)</f>
         <v>3809000</v>
       </c>
-      <c r="F35" s="20" t="n">
-        <f aca="false">IF(B35=0,0,1-C35/B35)</f>
+      <c r="F44" s="24" t="n">
+        <f aca="false">IF(B44=0,0,1-C44/B44)</f>
         <v>0.306719099969636</v>
       </c>
-      <c r="G35" s="20" t="n">
-        <f aca="false">IF(B35=0,0,1-D35/B35)</f>
+      <c r="G44" s="24" t="n">
+        <f aca="false">IF(B44=0,0,1-D44/B44)</f>
         <v>0.468949919899944</v>
       </c>
-      <c r="H35" s="21" t="n">
-        <f aca="false">IF(C35=0,0,(E35-C35)/C35)</f>
+      <c r="H44" s="25" t="n">
+        <f aca="false">IF(C44=0,0,(E44-C44)/C44)</f>
         <v>-0.2704332953409</v>
       </c>
-      <c r="I35" s="21" t="n">
-        <f aca="false">IF(D35=0,0,(E35-D35)/D35)</f>
+      <c r="I44" s="25" t="n">
+        <f aca="false">IF(D44=0,0,(E44-D44)/D44)</f>
         <v>-0.047557508054703</v>
       </c>
     </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A38" s="12" t="s">
-        <v>66</v>
-      </c>
-      <c r="B38" s="12"/>
-      <c r="C38" s="12"/>
-      <c r="D38" s="12"/>
-      <c r="E38" s="12"/>
-      <c r="F38" s="12"/>
-      <c r="G38" s="12"/>
-      <c r="H38" s="12"/>
-      <c r="I38" s="12"/>
-    </row>
-    <row r="39" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A39" s="3" t="s">
-        <v>67</v>
-      </c>
-      <c r="B39" s="3" t="s">
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A47" s="12" t="s">
+        <v>69</v>
+      </c>
+      <c r="B47" s="12"/>
+      <c r="C47" s="12"/>
+      <c r="D47" s="12"/>
+      <c r="E47" s="12"/>
+      <c r="F47" s="12"/>
+      <c r="G47" s="12"/>
+      <c r="H47" s="12"/>
+      <c r="I47" s="12"/>
+    </row>
+    <row r="48" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A48" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="B48" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="C39" s="3" t="s">
+      <c r="C48" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="D39" s="3" t="s">
+      <c r="D48" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="E39" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="F39" s="3" t="s">
-        <v>69</v>
-      </c>
-    </row>
-    <row r="40" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A40" s="24" t="s">
-        <v>70</v>
-      </c>
-      <c r="B40" s="14" t="n">
+      <c r="E48" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="F48" s="3" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A49" s="27" t="s">
+        <v>73</v>
+      </c>
+      <c r="B49" s="14" t="n">
         <v>5858217.9075</v>
       </c>
-      <c r="C40" s="14" t="n">
+      <c r="C49" s="14" t="n">
         <v>3665191.82106667</v>
       </c>
-      <c r="D40" s="14" t="n">
+      <c r="D49" s="14" t="n">
         <v>3665191.82106667</v>
       </c>
-      <c r="E40" s="14" t="n">
-        <f aca="false">B40-C40</f>
+      <c r="E49" s="14" t="n">
+        <f aca="false">B49-C49</f>
         <v>2193026.08643333</v>
       </c>
-      <c r="F40" s="14" t="n">
-        <f aca="false">B40-D40</f>
+      <c r="F49" s="14" t="n">
+        <f aca="false">B49-D49</f>
         <v>2193026.08643333</v>
       </c>
     </row>
-    <row r="41" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A41" s="24" t="s">
+    <row r="50" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A50" s="27" t="s">
         <v>27</v>
       </c>
-      <c r="B41" s="14" t="n">
+      <c r="B50" s="14" t="n">
         <v>1593669.9975</v>
       </c>
-      <c r="C41" s="14" t="n">
+      <c r="C50" s="14" t="n">
         <v>1476879.195</v>
       </c>
-      <c r="D41" s="14" t="n">
+      <c r="D50" s="14" t="n">
         <v>255163.665</v>
       </c>
-      <c r="E41" s="14" t="n">
-        <f aca="false">B41-C41</f>
+      <c r="E50" s="14" t="n">
+        <f aca="false">B50-C50</f>
         <v>116790.8025</v>
       </c>
-      <c r="F41" s="14" t="n">
-        <f aca="false">B41-D41</f>
+      <c r="F50" s="14" t="n">
+        <f aca="false">B50-D50</f>
         <v>1338506.3325</v>
       </c>
     </row>
-    <row r="42" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A42" s="24" t="s">
-        <v>71</v>
-      </c>
-      <c r="B42" s="14" t="n">
+    <row r="51" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A51" s="27" t="s">
+        <v>74</v>
+      </c>
+      <c r="B51" s="14" t="n">
         <v>78836.1</v>
       </c>
-      <c r="C42" s="14" t="n">
+      <c r="C51" s="14" t="n">
         <v>78836.1</v>
       </c>
-      <c r="D42" s="14" t="n">
+      <c r="D51" s="14" t="n">
         <v>78836.1</v>
       </c>
-      <c r="E42" s="14" t="n">
-        <f aca="false">B42-C42</f>
-        <v>0</v>
-      </c>
-      <c r="F42" s="14" t="n">
-        <f aca="false">B42-D42</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="43" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A43" s="10" t="s">
-        <v>53</v>
-      </c>
-      <c r="B43" s="19" t="n">
-        <f aca="false">SUM(B40:B42)</f>
+      <c r="E51" s="14" t="n">
+        <f aca="false">B51-C51</f>
+        <v>0</v>
+      </c>
+      <c r="F51" s="14" t="n">
+        <f aca="false">B51-D51</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A52" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="B52" s="23" t="n">
+        <f aca="false">SUM(B49:B51)</f>
         <v>7530724.005</v>
       </c>
-      <c r="C43" s="19" t="n">
-        <f aca="false">SUM(C40:C42)</f>
+      <c r="C52" s="23" t="n">
+        <f aca="false">SUM(C49:C51)</f>
         <v>5220907.11606667</v>
       </c>
-      <c r="D43" s="19" t="n">
-        <f aca="false">SUM(D40:D42)</f>
+      <c r="D52" s="23" t="n">
+        <f aca="false">SUM(D49:D51)</f>
         <v>3999191.58606667</v>
       </c>
-      <c r="E43" s="19" t="n">
-        <f aca="false">SUM(E40:E42)</f>
+      <c r="E52" s="23" t="n">
+        <f aca="false">SUM(E49:E51)</f>
         <v>2309816.88893333</v>
       </c>
-      <c r="F43" s="19" t="n">
-        <f aca="false">SUM(F40:F42)</f>
+      <c r="F52" s="23" t="n">
+        <f aca="false">SUM(F49:F51)</f>
         <v>3531532.41893333</v>
       </c>
     </row>
-    <row r="45" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A45" s="2" t="s">
-        <v>72</v>
+    <row r="54" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A54" s="2" t="s">
+        <v>75</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="4">
     <mergeCell ref="A2:I2"/>
-    <mergeCell ref="A13:I13"/>
-    <mergeCell ref="A26:I26"/>
-    <mergeCell ref="A38:I38"/>
+    <mergeCell ref="A16:I16"/>
+    <mergeCell ref="A32:I32"/>
+    <mergeCell ref="A47:I47"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>

<commit_message>
Use the agreed S1 scope basis alignment justification
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016KmKbhNhfEuuXeBfiH8ZpM
</commit_message>
<xml_diff>
--- a/NMMP_Reductions_Nuclear_Pharma.xlsx
+++ b/NMMP_Reductions_Nuclear_Pharma.xlsx
@@ -23,7 +23,7 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="76">
   <si>
-    <t xml:space="preserve">Reductions on the NMMP offer — all amounts in AUD. Nuclear reductions are applied in sequence, without double counting: SSC descoping → S1 deliverable adjustment → rework → travel → management overlap adjustment (4%). Plan Safe applies to Scenario 2 only.</t>
+    <t xml:space="preserve">Reductions on the NMMP offer — all amounts in AUD. Nuclear reductions are applied in sequence, without double counting: SSC descoping → S1 scope basis alignment → rework → travel → management overlap adjustment (4%). Plan Safe applies to Scenario 2 only.</t>
   </si>
   <si>
     <t xml:space="preserve">Discipline</t>
@@ -89,10 +89,10 @@
     <t xml:space="preserve">All</t>
   </si>
   <si>
-    <t xml:space="preserve">S1 deliverable adjustment</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Safety Assurance Plan / Safety Integration Plan priced as two weeks of work: a single, unrevised issue in Stage 1 of 190 hours and 44,559 AUD (2.5 FTEs full time for two weeks). The Stage 2 update is removed. Original price 432,419 AUD − 44,559 AUD.</t>
+    <t xml:space="preserve">S1 – Safety Assurance / Integration Plan – Scope Basis Alignment</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The original allowance for S1 was based on the assumption that the Safety Assurance / Safety Integration framework would be developed and maintained through Stages 1 and 2, including the initial preparation, definition of methodologies and interfaces, coordination with the relevant design parties, incorporation of project developments and subsequent updates/re-issues as the design progressed. Following Synertec’s clarification on the expected scope and timing of this deliverable, the revised allowance is based on a limited initial activity of 2.5 FTE for two weeks, covering the preparation, coordination, internal review and initial issue of the S1 deliverable. No subsequent development, maintenance, updates, re-issues or ongoing safety assurance/integration support beyond this initial two-week period are included; any such activities, if subsequently required, would be subject to separate agreement.</t>
   </si>
   <si>
     <t xml:space="preserve">S1</t>

</xml_diff>

<commit_message>
Use the agreed travel justification
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016KmKbhNhfEuuXeBfiH8ZpM
</commit_message>
<xml_diff>
--- a/NMMP_Reductions_Nuclear_Pharma.xlsx
+++ b/NMMP_Reductions_Nuclear_Pharma.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="76">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="77">
   <si>
     <t xml:space="preserve">Reductions on the NMMP offer — all amounts in AUD. Nuclear reductions are applied in sequence, without double counting: SSC descoping → S1 scope basis alignment → rework → travel → management overlap adjustment (4%). Plan Safe applies to Scenario 2 only.</t>
   </si>
@@ -102,6 +102,9 @@
   </si>
   <si>
     <t xml:space="preserve">Travel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The original offer included an allowance for potential travel to Australia during project execution. This allowance has been removed from the revised price. No travel is included in the revised commercial proposal; any travel required by Synertec, ANSTO or the project needs will be agreed in advance and charged separately, including the applicable travel expenses and travel time.</t>
   </si>
   <si>
     <t xml:space="preserve">Plan Safe</t>
@@ -942,9 +945,8 @@
       <c r="D7" s="5" t="n">
         <v>70000</v>
       </c>
-      <c r="E7" s="6" t="str">
-        <f aca="false">"Travel allowance removed: 70,000 AUD."</f>
-        <v>Travel allowance removed: 70,000 AUD.</v>
+      <c r="E7" s="6" t="s">
+        <v>27</v>
       </c>
       <c r="F7" s="7" t="s">
         <v>12</v>
@@ -964,7 +966,7 @@
         <v>6</v>
       </c>
       <c r="C8" s="7" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D8" s="5" t="n">
         <v>1221715.53</v>
@@ -974,36 +976,36 @@
         <v>Plan Safe's own human factors deliverables removed (HF Assurance / Integration Plan, HF Hazards Identification and Control Plan, HF Task Assessments, HF Substantiation Report). Value = their price in the original offer. Plan Safe keeps its share of the shared deliverables.</v>
       </c>
       <c r="F8" s="7" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="G8" s="7" t="s">
         <v>18</v>
       </c>
       <c r="H8" s="7" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B9" s="7" t="n">
         <v>7</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="D9" s="9"/>
       <c r="E9" s="8"/>
       <c r="F9" s="8"/>
       <c r="G9" s="8"/>
       <c r="H9" s="7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B10" s="7" t="n">
         <v>8</v>
@@ -1014,12 +1016,12 @@
       <c r="F10" s="8"/>
       <c r="G10" s="8"/>
       <c r="H10" s="7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B11" s="7" t="n">
         <v>9</v>
@@ -1030,12 +1032,12 @@
       <c r="F11" s="8"/>
       <c r="G11" s="8"/>
       <c r="H11" s="7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B12" s="7" t="n">
         <v>10</v>
@@ -1046,12 +1048,12 @@
       <c r="F12" s="8"/>
       <c r="G12" s="8"/>
       <c r="H12" s="7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B13" s="7" t="n">
         <v>11</v>
@@ -1062,12 +1064,12 @@
       <c r="F13" s="8"/>
       <c r="G13" s="8"/>
       <c r="H13" s="7" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C15" s="10" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D15" s="11" t="n">
         <f aca="false">SUM(D3:D7)</f>
@@ -1076,7 +1078,7 @@
     </row>
     <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C16" s="10" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D16" s="11" t="n">
         <f aca="false">SUM(D3:D8)</f>
@@ -1085,7 +1087,7 @@
     </row>
     <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C17" s="10" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D17" s="11" t="n">
         <f aca="false">SUM(D9:D13)</f>
@@ -1094,12 +1096,12 @@
     </row>
     <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
   </sheetData>
@@ -1131,7 +1133,7 @@
   <sheetData>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="12" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B2" s="12"/>
       <c r="C2" s="12"/>
@@ -1144,31 +1146,31 @@
     </row>
     <row r="3" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1239,7 +1241,7 @@
     </row>
     <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B6" s="14" t="n">
         <v>1469323.8</v>
@@ -1272,7 +1274,7 @@
     </row>
     <row r="7" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="18" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B7" s="19" t="n">
         <f aca="false">N(B4)+N(B5)+N(B6)</f>
@@ -1309,7 +1311,7 @@
     </row>
     <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="13" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B8" s="14" t="n">
         <v>3183882.555</v>
@@ -1342,7 +1344,7 @@
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="13" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B9" s="14" t="n">
         <v>540610.875</v>
@@ -1375,7 +1377,7 @@
     </row>
     <row r="10" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="18" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B10" s="19" t="n">
         <f aca="false">N(B8)+N(B9)</f>
@@ -1412,7 +1414,7 @@
     </row>
     <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="13" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B11" s="14" t="n">
         <v>775079.55</v>
@@ -1445,7 +1447,7 @@
     </row>
     <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="13" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B12" s="14" t="n">
         <v>493905.3</v>
@@ -1478,7 +1480,7 @@
     </row>
     <row r="13" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="18" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B13" s="19" t="n">
         <f aca="false">N(B11)+N(B12)</f>
@@ -1515,7 +1517,7 @@
     </row>
     <row r="14" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="22" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B14" s="23" t="n">
         <f aca="false">N(B4)+N(B5)+N(B6)+N(B8)+N(B9)+N(B11)+N(B12)</f>
@@ -1552,7 +1554,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="12" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B16" s="12"/>
       <c r="C16" s="12"/>
@@ -1565,25 +1567,25 @@
     </row>
     <row r="17" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="3" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="G17" s="3" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1628,7 +1630,7 @@
     </row>
     <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="13" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B20" s="26"/>
       <c r="C20" s="26"/>
@@ -1648,7 +1650,7 @@
     </row>
     <row r="21" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="18" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B21" s="19" t="n">
         <f aca="false">N(B18)+N(B19)+N(B20)</f>
@@ -1677,7 +1679,7 @@
     </row>
     <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="13" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B22" s="26"/>
       <c r="C22" s="26"/>
@@ -1697,7 +1699,7 @@
     </row>
     <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="13" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B23" s="26"/>
       <c r="C23" s="26"/>
@@ -1717,7 +1719,7 @@
     </row>
     <row r="24" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="18" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B24" s="19" t="n">
         <f aca="false">N(B22)+N(B23)</f>
@@ -1746,7 +1748,7 @@
     </row>
     <row r="25" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="13" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B25" s="26"/>
       <c r="C25" s="26"/>
@@ -1766,7 +1768,7 @@
     </row>
     <row r="26" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="13" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B26" s="26"/>
       <c r="C26" s="26"/>
@@ -1786,7 +1788,7 @@
     </row>
     <row r="27" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="18" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B27" s="19" t="n">
         <f aca="false">N(B25)+N(B26)</f>
@@ -1815,7 +1817,7 @@
     </row>
     <row r="28" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="22" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B28" s="23" t="n">
         <f aca="false">N(B18)+N(B19)+N(B20)+N(B22)+N(B23)+N(B25)+N(B26)</f>
@@ -1850,12 +1852,12 @@
     </row>
     <row r="30" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="12" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B32" s="12"/>
       <c r="C32" s="12"/>
@@ -1868,31 +1870,31 @@
     </row>
     <row r="33" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="3" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="D33" s="3" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E33" s="3" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="F33" s="3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="G33" s="3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="H33" s="3" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="I33" s="3" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1971,7 +1973,7 @@
     </row>
     <row r="36" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="13" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="B36" s="14" t="n">
         <f aca="false">B6+N(B20)</f>
@@ -2008,7 +2010,7 @@
     </row>
     <row r="37" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="18" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B37" s="19" t="n">
         <f aca="false">N(B34)+N(B35)+N(B36)</f>
@@ -2045,7 +2047,7 @@
     </row>
     <row r="38" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="13" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B38" s="14" t="n">
         <f aca="false">B8+N(B22)</f>
@@ -2082,7 +2084,7 @@
     </row>
     <row r="39" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="13" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B39" s="14" t="n">
         <f aca="false">B9+N(B23)</f>
@@ -2119,7 +2121,7 @@
     </row>
     <row r="40" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="18" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B40" s="19" t="n">
         <f aca="false">N(B38)+N(B39)</f>
@@ -2156,7 +2158,7 @@
     </row>
     <row r="41" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="13" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B41" s="14" t="n">
         <f aca="false">B11+N(B25)</f>
@@ -2193,7 +2195,7 @@
     </row>
     <row r="42" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="13" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B42" s="14" t="n">
         <f aca="false">B12+N(B26)</f>
@@ -2230,7 +2232,7 @@
     </row>
     <row r="43" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="18" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B43" s="19" t="n">
         <f aca="false">N(B41)+N(B42)</f>
@@ -2267,7 +2269,7 @@
     </row>
     <row r="44" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="22" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B44" s="23" t="n">
         <f aca="false">N(B34)+N(B35)+N(B36)+N(B38)+N(B39)+N(B41)+N(B42)</f>
@@ -2304,7 +2306,7 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="12" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B47" s="12"/>
       <c r="C47" s="12"/>
@@ -2317,27 +2319,27 @@
     </row>
     <row r="48" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="3" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B48" s="3" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C48" s="3" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D48" s="3" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="E48" s="3" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="F48" s="3" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="27" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B49" s="14" t="n">
         <v>5858217.9075</v>
@@ -2359,7 +2361,7 @@
     </row>
     <row r="50" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="27" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B50" s="14" t="n">
         <v>1593669.9975</v>
@@ -2381,7 +2383,7 @@
     </row>
     <row r="51" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="27" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B51" s="14" t="n">
         <v>78836.1</v>
@@ -2403,7 +2405,7 @@
     </row>
     <row r="52" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="10" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B52" s="23" t="n">
         <f aca="false">SUM(B49:B51)</f>
@@ -2428,7 +2430,7 @@
     </row>
     <row r="54" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="2" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Use the agreed Plan Safe justification
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016KmKbhNhfEuuXeBfiH8ZpM
</commit_message>
<xml_diff>
--- a/NMMP_Reductions_Nuclear_Pharma.xlsx
+++ b/NMMP_Reductions_Nuclear_Pharma.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="78">
   <si>
     <t xml:space="preserve">Reductions on the NMMP offer — all amounts in AUD. Nuclear reductions are applied in sequence, without double counting: SSC descoping → S1 scope basis alignment → rework → travel → management overlap adjustment (4%). Plan Safe applies to Scenario 2 only.</t>
   </si>
@@ -108,6 +108,9 @@
   </si>
   <si>
     <t xml:space="preserve">Plan Safe</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The original Nuclear &amp; Radiological commercial envelope included an allowance for the specialist subcontractor scope in order to provide a complete tender price. In line with the subcontracting model contemplated in the MoU, IDOM proposes to remove the PlanSafe-only deliverables (S2, S3, S8 and S30) from its revised commercial scope. These activities would therefore be contracted and commercially agreed directly by Synertec with the relevant specialist subcontractor, with the corresponding scope, resourcing and commercial terms to be agreed between those parties.</t>
   </si>
   <si>
     <t xml:space="preserve">S2, S3, S8, S30</t>
@@ -971,41 +974,40 @@
       <c r="D8" s="5" t="n">
         <v>1221715.53</v>
       </c>
-      <c r="E8" s="6" t="str">
-        <f aca="false">"Plan Safe's own human factors deliverables removed (HF Assurance / Integration Plan, HF Hazards Identification and Control Plan, HF Task Assessments, HF Substantiation Report). Value = their price in the original offer. Plan Safe keeps its share of the shared deliverables."</f>
-        <v>Plan Safe's own human factors deliverables removed (HF Assurance / Integration Plan, HF Hazards Identification and Control Plan, HF Task Assessments, HF Substantiation Report). Value = their price in the original offer. Plan Safe keeps its share of the shared deliverables.</v>
+      <c r="E8" s="6" t="s">
+        <v>29</v>
       </c>
       <c r="F8" s="7" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="G8" s="7" t="s">
         <v>18</v>
       </c>
       <c r="H8" s="7" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B9" s="7" t="n">
         <v>7</v>
       </c>
       <c r="C9" s="8" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D9" s="9"/>
       <c r="E9" s="8"/>
       <c r="F9" s="8"/>
       <c r="G9" s="8"/>
       <c r="H9" s="7" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B10" s="7" t="n">
         <v>8</v>
@@ -1016,12 +1018,12 @@
       <c r="F10" s="8"/>
       <c r="G10" s="8"/>
       <c r="H10" s="7" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B11" s="7" t="n">
         <v>9</v>
@@ -1032,12 +1034,12 @@
       <c r="F11" s="8"/>
       <c r="G11" s="8"/>
       <c r="H11" s="7" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B12" s="7" t="n">
         <v>10</v>
@@ -1048,12 +1050,12 @@
       <c r="F12" s="8"/>
       <c r="G12" s="8"/>
       <c r="H12" s="7" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B13" s="7" t="n">
         <v>11</v>
@@ -1064,12 +1066,12 @@
       <c r="F13" s="8"/>
       <c r="G13" s="8"/>
       <c r="H13" s="7" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C15" s="10" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D15" s="11" t="n">
         <f aca="false">SUM(D3:D7)</f>
@@ -1078,7 +1080,7 @@
     </row>
     <row r="16" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C16" s="10" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D16" s="11" t="n">
         <f aca="false">SUM(D3:D8)</f>
@@ -1087,7 +1089,7 @@
     </row>
     <row r="17" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="C17" s="10" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="D17" s="11" t="n">
         <f aca="false">SUM(D9:D13)</f>
@@ -1096,12 +1098,12 @@
     </row>
     <row r="19" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
   </sheetData>
@@ -1133,7 +1135,7 @@
   <sheetData>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="12" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B2" s="12"/>
       <c r="C2" s="12"/>
@@ -1146,31 +1148,31 @@
     </row>
     <row r="3" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1241,7 +1243,7 @@
     </row>
     <row r="6" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B6" s="14" t="n">
         <v>1469323.8</v>
@@ -1274,7 +1276,7 @@
     </row>
     <row r="7" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="18" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B7" s="19" t="n">
         <f aca="false">N(B4)+N(B5)+N(B6)</f>
@@ -1311,7 +1313,7 @@
     </row>
     <row r="8" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="13" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B8" s="14" t="n">
         <v>3183882.555</v>
@@ -1344,7 +1346,7 @@
     </row>
     <row r="9" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="13" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B9" s="14" t="n">
         <v>540610.875</v>
@@ -1377,7 +1379,7 @@
     </row>
     <row r="10" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="18" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B10" s="19" t="n">
         <f aca="false">N(B8)+N(B9)</f>
@@ -1414,7 +1416,7 @@
     </row>
     <row r="11" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="13" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B11" s="14" t="n">
         <v>775079.55</v>
@@ -1447,7 +1449,7 @@
     </row>
     <row r="12" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="13" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B12" s="14" t="n">
         <v>493905.3</v>
@@ -1480,7 +1482,7 @@
     </row>
     <row r="13" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="18" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B13" s="19" t="n">
         <f aca="false">N(B11)+N(B12)</f>
@@ -1517,7 +1519,7 @@
     </row>
     <row r="14" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="22" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B14" s="23" t="n">
         <f aca="false">N(B4)+N(B5)+N(B6)+N(B8)+N(B9)+N(B11)+N(B12)</f>
@@ -1554,7 +1556,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="12" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B16" s="12"/>
       <c r="C16" s="12"/>
@@ -1567,25 +1569,25 @@
     </row>
     <row r="17" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="3" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E17" s="3" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="F17" s="3" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="G17" s="3" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1630,7 +1632,7 @@
     </row>
     <row r="20" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="13" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B20" s="26"/>
       <c r="C20" s="26"/>
@@ -1650,7 +1652,7 @@
     </row>
     <row r="21" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="18" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B21" s="19" t="n">
         <f aca="false">N(B18)+N(B19)+N(B20)</f>
@@ -1679,7 +1681,7 @@
     </row>
     <row r="22" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="13" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B22" s="26"/>
       <c r="C22" s="26"/>
@@ -1699,7 +1701,7 @@
     </row>
     <row r="23" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="13" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B23" s="26"/>
       <c r="C23" s="26"/>
@@ -1719,7 +1721,7 @@
     </row>
     <row r="24" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="18" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B24" s="19" t="n">
         <f aca="false">N(B22)+N(B23)</f>
@@ -1748,7 +1750,7 @@
     </row>
     <row r="25" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="13" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B25" s="26"/>
       <c r="C25" s="26"/>
@@ -1768,7 +1770,7 @@
     </row>
     <row r="26" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="13" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B26" s="26"/>
       <c r="C26" s="26"/>
@@ -1788,7 +1790,7 @@
     </row>
     <row r="27" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="18" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B27" s="19" t="n">
         <f aca="false">N(B25)+N(B26)</f>
@@ -1817,7 +1819,7 @@
     </row>
     <row r="28" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="22" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B28" s="23" t="n">
         <f aca="false">N(B18)+N(B19)+N(B20)+N(B22)+N(B23)+N(B25)+N(B26)</f>
@@ -1852,12 +1854,12 @@
     </row>
     <row r="30" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="12" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B32" s="12"/>
       <c r="C32" s="12"/>
@@ -1870,31 +1872,31 @@
     </row>
     <row r="33" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="3" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B33" s="3" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D33" s="3" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E33" s="3" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="F33" s="3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="G33" s="3" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="H33" s="3" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="I33" s="3" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -1973,7 +1975,7 @@
     </row>
     <row r="36" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="13" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B36" s="14" t="n">
         <f aca="false">B6+N(B20)</f>
@@ -2010,7 +2012,7 @@
     </row>
     <row r="37" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="18" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B37" s="19" t="n">
         <f aca="false">N(B34)+N(B35)+N(B36)</f>
@@ -2047,7 +2049,7 @@
     </row>
     <row r="38" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="13" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B38" s="14" t="n">
         <f aca="false">B8+N(B22)</f>
@@ -2084,7 +2086,7 @@
     </row>
     <row r="39" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="13" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="B39" s="14" t="n">
         <f aca="false">B9+N(B23)</f>
@@ -2121,7 +2123,7 @@
     </row>
     <row r="40" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="18" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B40" s="19" t="n">
         <f aca="false">N(B38)+N(B39)</f>
@@ -2158,7 +2160,7 @@
     </row>
     <row r="41" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="13" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B41" s="14" t="n">
         <f aca="false">B11+N(B25)</f>
@@ -2195,7 +2197,7 @@
     </row>
     <row r="42" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="13" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B42" s="14" t="n">
         <f aca="false">B12+N(B26)</f>
@@ -2232,7 +2234,7 @@
     </row>
     <row r="43" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="18" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B43" s="19" t="n">
         <f aca="false">N(B41)+N(B42)</f>
@@ -2269,7 +2271,7 @@
     </row>
     <row r="44" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="22" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B44" s="23" t="n">
         <f aca="false">N(B34)+N(B35)+N(B36)+N(B38)+N(B39)+N(B41)+N(B42)</f>
@@ -2306,7 +2308,7 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="12" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="B47" s="12"/>
       <c r="C47" s="12"/>
@@ -2319,27 +2321,27 @@
     </row>
     <row r="48" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="3" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B48" s="3" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C48" s="3" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D48" s="3" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="E48" s="3" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="F48" s="3" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="27" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="B49" s="14" t="n">
         <v>5858217.9075</v>
@@ -2383,7 +2385,7 @@
     </row>
     <row r="51" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="27" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B51" s="14" t="n">
         <v>78836.1</v>
@@ -2405,7 +2407,7 @@
     </row>
     <row r="52" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A52" s="10" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B52" s="23" t="n">
         <f aca="false">SUM(B49:B51)</f>
@@ -2430,7 +2432,7 @@
     </row>
     <row r="54" customFormat="false" ht="14.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="2" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
     </row>
   </sheetData>

</xml_diff>